<commit_message>
Add Review Flag column for unmatched/case-insensitive BOM rows
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4gmyWjX7HwofLtwBHfu93
</commit_message>
<xml_diff>
--- a/Krayden_Europe_-_Bill_of_Materials_Transformed.xlsx
+++ b/Krayden_Europe_-_Bill_of_Materials_Transformed.xlsx
@@ -760,7 +760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I380"/>
+  <dimension ref="A1:J380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="11" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -771,7 +771,7 @@
     <col width="31.7109375" bestFit="1" customWidth="1" style="5" min="7" max="7"/>
     <col width="22.7109375" bestFit="1" customWidth="1" style="5" min="8" max="8"/>
     <col width="16.140625" bestFit="1" customWidth="1" style="5" min="9" max="9"/>
-    <col width="9.140625" customWidth="1" style="5" min="10" max="10"/>
+    <col width="60" customWidth="1" style="5" min="10" max="10"/>
     <col width="9.140625" customWidth="1" style="5" min="11" max="16384"/>
   </cols>
   <sheetData>
@@ -821,6 +821,11 @@
           <t>Include Children</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Review Flag</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1066,6 +1071,11 @@
       <c r="I8" s="14" t="b">
         <v>1</v>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Matched to product report ignoring case (GDL1850/40x40) - verify</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
@@ -2154,6 +2164,11 @@
       </c>
       <c r="I41" s="14" t="b">
         <v>1</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>No match in product data report - name not updated</t>
+        </is>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
Set BOM Revision names to Rev 1
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4gmyWjX7HwofLtwBHfu93
</commit_message>
<xml_diff>
--- a/Krayden_Europe_-_Bill_of_Materials_Transformed.xlsx
+++ b/Krayden_Europe_-_Bill_of_Materials_Transformed.xlsx
@@ -13466,7 +13466,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>GDL2200/C11.3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -13487,7 +13487,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>GDL2900/C5.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -13508,7 +13508,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>GDL1500/C11.3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -13529,7 +13529,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>GDL1500/6X6R4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -13550,7 +13550,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>GDL1850/40X40 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -13571,7 +13571,7 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>MREC909/A67C Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
@@ -13592,7 +13592,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.350 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
@@ -13613,7 +13613,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>TR7/SAC305/0.457 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -13634,7 +13634,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.457 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
@@ -13655,7 +13655,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.300 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -13676,7 +13676,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.250 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
@@ -13697,7 +13697,7 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.350T Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -13718,7 +13718,7 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>TR13-Sn63Pb37/0.560 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -13739,7 +13739,7 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>TR7/SAC305/0.300 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
@@ -13760,7 +13760,7 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.500 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
@@ -13781,7 +13781,7 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>TR7/SAC305/0.500 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
@@ -13802,7 +13802,7 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>TR7-Bi58Sn42/0.300 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
@@ -13823,7 +13823,7 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>TR7-Bi58Sn42/0.500 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
@@ -13844,7 +13844,7 @@
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>TR13-Bi58Sn42/0.300 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
@@ -13865,7 +13865,7 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>TR13-Bi58Sn42/0.500 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -13886,7 +13886,7 @@
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>TR7/SAC305/0.400 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -13907,7 +13907,7 @@
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.400 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -13928,7 +13928,7 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC105/0.300 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
@@ -13949,7 +13949,7 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>TR13-CCSAC305/0.350 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -13970,7 +13970,7 @@
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>TR13-Sn10Pb90/0.380 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
@@ -13991,7 +13991,7 @@
       </c>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>TR13-Sn10Pb90/0.500 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C29" s="14" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.600 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C30" s="14" t="inlineStr">
@@ -14033,7 +14033,7 @@
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>TR13-SAC305/0.760-30kpcs Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C31" s="14" t="inlineStr">
@@ -14054,7 +14054,7 @@
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
@@ -14075,7 +14075,7 @@
       </c>
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/12 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C33" s="14" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -14117,7 +14117,7 @@
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C35" s="14" t="inlineStr">
@@ -14138,7 +14138,7 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -14159,7 +14159,7 @@
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/20 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C37" s="14" t="inlineStr">
@@ -14180,7 +14180,7 @@
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/25 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
@@ -14201,7 +14201,7 @@
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -14222,7 +14222,7 @@
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
@@ -14243,7 +14243,7 @@
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/101 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -14264,7 +14264,7 @@
       </c>
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr">
@@ -14285,7 +14285,7 @@
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr">
@@ -14306,7 +14306,7 @@
       </c>
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/12 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr">
@@ -14327,7 +14327,7 @@
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C45" s="14" t="inlineStr">
@@ -14348,7 +14348,7 @@
       </c>
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C46" s="14" t="inlineStr">
@@ -14369,7 +14369,7 @@
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/20 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C47" s="14" t="inlineStr">
@@ -14390,7 +14390,7 @@
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/25 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C48" s="14" t="inlineStr">
@@ -14411,7 +14411,7 @@
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C49" s="14" t="inlineStr">
@@ -14432,7 +14432,7 @@
       </c>
       <c r="B50" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="B51" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C51" s="14" t="inlineStr">
@@ -14474,7 +14474,7 @@
       </c>
       <c r="B52" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/200 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C52" s="14" t="inlineStr">
@@ -14495,7 +14495,7 @@
       </c>
       <c r="B53" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C53" s="14" t="inlineStr">
@@ -14516,7 +14516,7 @@
       </c>
       <c r="B54" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C54" s="14" t="inlineStr">
@@ -14537,7 +14537,7 @@
       </c>
       <c r="B55" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/12 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C55" s="14" t="inlineStr">
@@ -14558,7 +14558,7 @@
       </c>
       <c r="B56" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C56" s="14" t="inlineStr">
@@ -14579,7 +14579,7 @@
       </c>
       <c r="B57" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C57" s="14" t="inlineStr">
@@ -14600,7 +14600,7 @@
       </c>
       <c r="B58" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/20 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C58" s="14" t="inlineStr">
@@ -14621,7 +14621,7 @@
       </c>
       <c r="B59" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/25 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C59" s="14" t="inlineStr">
@@ -14642,7 +14642,7 @@
       </c>
       <c r="B60" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C60" s="14" t="inlineStr">
@@ -14663,7 +14663,7 @@
       </c>
       <c r="B61" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C61" s="14" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="B62" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C62" s="14" t="inlineStr">
@@ -14705,7 +14705,7 @@
       </c>
       <c r="B63" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C63" s="14" t="inlineStr">
@@ -14726,7 +14726,7 @@
       </c>
       <c r="B64" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C64" s="14" t="inlineStr">
@@ -14747,7 +14747,7 @@
       </c>
       <c r="B65" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/12 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C65" s="14" t="inlineStr">
@@ -14768,7 +14768,7 @@
       </c>
       <c r="B66" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C66" s="14" t="inlineStr">
@@ -14789,7 +14789,7 @@
       </c>
       <c r="B67" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C67" s="14" t="inlineStr">
@@ -14810,7 +14810,7 @@
       </c>
       <c r="B68" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/20 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C68" s="14" t="inlineStr">
@@ -14831,7 +14831,7 @@
       </c>
       <c r="B69" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/25 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C69" s="14" t="inlineStr">
@@ -14852,7 +14852,7 @@
       </c>
       <c r="B70" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C70" s="14" t="inlineStr">
@@ -14873,7 +14873,7 @@
       </c>
       <c r="B71" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C71" s="14" t="inlineStr">
@@ -14894,7 +14894,7 @@
       </c>
       <c r="B72" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C72" s="14" t="inlineStr">
@@ -14915,7 +14915,7 @@
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>PIT2SD/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C73" s="14" t="inlineStr">
@@ -14936,7 +14936,7 @@
       </c>
       <c r="B74" s="13" t="inlineStr">
         <is>
-          <t>PIT2SD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C74" s="14" t="inlineStr">
@@ -14957,7 +14957,7 @@
       </c>
       <c r="B75" s="13" t="inlineStr">
         <is>
-          <t>PIT2SD/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C75" s="14" t="inlineStr">
@@ -14978,7 +14978,7 @@
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t>PIT2SD/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C76" s="14" t="inlineStr">
@@ -14999,7 +14999,7 @@
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
-          <t>PIT2SD/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C77" s="14" t="inlineStr">
@@ -15020,7 +15020,7 @@
       </c>
       <c r="B78" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C78" s="14" t="inlineStr">
@@ -15041,7 +15041,7 @@
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C79" s="14" t="inlineStr">
@@ -15062,7 +15062,7 @@
       </c>
       <c r="B80" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C80" s="14" t="inlineStr">
@@ -15083,7 +15083,7 @@
       </c>
       <c r="B81" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C81" s="14" t="inlineStr">
@@ -15104,7 +15104,7 @@
       </c>
       <c r="B82" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C82" s="14" t="inlineStr">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-WL-SG/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
@@ -15146,7 +15146,7 @@
       </c>
       <c r="B84" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-WL-SG/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C84" s="14" t="inlineStr">
@@ -15167,7 +15167,7 @@
       </c>
       <c r="B85" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-WL-SG/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C85" s="14" t="inlineStr">
@@ -15188,7 +15188,7 @@
       </c>
       <c r="B86" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-WL-SG/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C86" s="14" t="inlineStr">
@@ -15209,7 +15209,7 @@
       </c>
       <c r="B87" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-WL-SG/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C87" s="14" t="inlineStr">
@@ -15230,7 +15230,7 @@
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>PET1S-Blue/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C88" s="14" t="inlineStr">
@@ -15251,7 +15251,7 @@
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
-          <t>PET1S-Blue/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C89" s="14" t="inlineStr">
@@ -15272,7 +15272,7 @@
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
-          <t>PET1S-Blue/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C90" s="14" t="inlineStr">
@@ -15293,7 +15293,7 @@
       </c>
       <c r="B91" s="13" t="inlineStr">
         <is>
-          <t>PET1S-Blue/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C91" s="14" t="inlineStr">
@@ -15314,7 +15314,7 @@
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
-          <t>PET1S-Blue/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C92" s="14" t="inlineStr">
@@ -15335,7 +15335,7 @@
       </c>
       <c r="B93" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C93" s="14" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="B94" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C94" s="14" t="inlineStr">
@@ -15377,7 +15377,7 @@
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C95" s="14" t="inlineStr">
@@ -15398,7 +15398,7 @@
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C96" s="14" t="inlineStr">
@@ -15419,7 +15419,7 @@
       </c>
       <c r="B97" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C97" s="14" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C98" s="14" t="inlineStr">
@@ -15461,7 +15461,7 @@
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C99" s="14" t="inlineStr">
@@ -15482,7 +15482,7 @@
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C100" s="14" t="inlineStr">
@@ -15503,7 +15503,7 @@
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C101" s="14" t="inlineStr">
@@ -15524,7 +15524,7 @@
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
@@ -15545,7 +15545,7 @@
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C103" s="14" t="inlineStr">
@@ -15566,7 +15566,7 @@
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/4.2 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C104" s="14" t="inlineStr">
@@ -15587,7 +15587,7 @@
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C105" s="14" t="inlineStr">
@@ -15608,7 +15608,7 @@
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/4.2 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C106" s="14" t="inlineStr">
@@ -15629,7 +15629,7 @@
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C107" s="14" t="inlineStr">
@@ -15650,7 +15650,7 @@
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C108" s="14" t="inlineStr">
@@ -15671,7 +15671,7 @@
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C109" s="14" t="inlineStr">
@@ -15692,7 +15692,7 @@
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C110" s="14" t="inlineStr">
@@ -15713,7 +15713,7 @@
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C111" s="14" t="inlineStr">
@@ -15734,7 +15734,7 @@
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
@@ -15755,7 +15755,7 @@
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>PIT5N/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C113" s="14" t="inlineStr">
@@ -15776,7 +15776,7 @@
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>PIT5N/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C114" s="14" t="inlineStr">
@@ -15797,7 +15797,7 @@
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
-          <t>PIT5N/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C115" s="14" t="inlineStr">
@@ -15818,7 +15818,7 @@
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
-          <t>PIT5N/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C116" s="14" t="inlineStr">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
-          <t>PIT5N/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C117" s="14" t="inlineStr">
@@ -15860,7 +15860,7 @@
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
-          <t>PIT5N/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C118" s="14" t="inlineStr">
@@ -15881,7 +15881,7 @@
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/150 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C119" s="14" t="inlineStr">
@@ -15902,7 +15902,7 @@
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C120" s="14" t="inlineStr">
@@ -15923,7 +15923,7 @@
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/101.6 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C121" s="14" t="inlineStr">
@@ -15944,7 +15944,7 @@
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/254 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
@@ -15965,7 +15965,7 @@
       </c>
       <c r="B123" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/304.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C123" s="14" t="inlineStr">
@@ -15986,7 +15986,7 @@
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/203.2 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C124" s="14" t="inlineStr">
@@ -16007,7 +16007,7 @@
       </c>
       <c r="B125" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C125" s="14" t="inlineStr">
@@ -16028,7 +16028,7 @@
       </c>
       <c r="B126" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/17.9 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C126" s="14" t="inlineStr">
@@ -16049,7 +16049,7 @@
       </c>
       <c r="B127" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C127" s="14" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="B128" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C128" s="14" t="inlineStr">
@@ -16091,7 +16091,7 @@
       </c>
       <c r="B129" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C129" s="14" t="inlineStr">
@@ -16112,7 +16112,7 @@
       </c>
       <c r="B130" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C130" s="14" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="B131" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C131" s="14" t="inlineStr">
@@ -16154,7 +16154,7 @@
       </c>
       <c r="B132" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-2RL/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C132" s="14" t="inlineStr">
@@ -16175,7 +16175,7 @@
       </c>
       <c r="B133" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-2RL/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C133" s="14" t="inlineStr">
@@ -16196,7 +16196,7 @@
       </c>
       <c r="B134" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-2RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C134" s="14" t="inlineStr">
@@ -16217,7 +16217,7 @@
       </c>
       <c r="B135" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-2RL/101.6 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C135" s="14" t="inlineStr">
@@ -16238,7 +16238,7 @@
       </c>
       <c r="B136" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/180 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C136" s="14" t="inlineStr">
@@ -16259,7 +16259,7 @@
       </c>
       <c r="B137" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/101.6 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C137" s="14" t="inlineStr">
@@ -16280,7 +16280,7 @@
       </c>
       <c r="B138" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C138" s="14" t="inlineStr">
@@ -16301,7 +16301,7 @@
       </c>
       <c r="B139" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C139" s="14" t="inlineStr">
@@ -16322,7 +16322,7 @@
       </c>
       <c r="B140" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C140" s="14" t="inlineStr">
@@ -16343,7 +16343,7 @@
       </c>
       <c r="B141" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C141" s="14" t="inlineStr">
@@ -16364,7 +16364,7 @@
       </c>
       <c r="B142" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C142" s="14" t="inlineStr">
@@ -16385,7 +16385,7 @@
       </c>
       <c r="B143" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C143" s="14" t="inlineStr">
@@ -16406,7 +16406,7 @@
       </c>
       <c r="B144" s="13" t="inlineStr">
         <is>
-          <t>PIT5N/96.5 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C144" s="14" t="inlineStr">
@@ -16427,7 +16427,7 @@
       </c>
       <c r="B145" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/40 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C145" s="14" t="inlineStr">
@@ -16448,7 +16448,7 @@
       </c>
       <c r="B146" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/127 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C146" s="14" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="B147" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/152 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C147" s="14" t="inlineStr">
@@ -16490,7 +16490,7 @@
       </c>
       <c r="B148" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/27 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C148" s="14" t="inlineStr">
@@ -16511,7 +16511,7 @@
       </c>
       <c r="B149" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/9 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C149" s="14" t="inlineStr">
@@ -16532,7 +16532,7 @@
       </c>
       <c r="B150" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/93 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C150" s="14" t="inlineStr">
@@ -16553,7 +16553,7 @@
       </c>
       <c r="B151" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/9.53 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C151" s="14" t="inlineStr">
@@ -16574,7 +16574,7 @@
       </c>
       <c r="B152" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C152" s="14" t="inlineStr">
@@ -16595,7 +16595,7 @@
       </c>
       <c r="B153" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C153" s="14" t="inlineStr">
@@ -16616,7 +16616,7 @@
       </c>
       <c r="B154" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C154" s="14" t="inlineStr">
@@ -16637,7 +16637,7 @@
       </c>
       <c r="B155" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C155" s="14" t="inlineStr">
@@ -16658,7 +16658,7 @@
       </c>
       <c r="B156" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C156" s="14" t="inlineStr">
@@ -16679,7 +16679,7 @@
       </c>
       <c r="B157" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/36.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C157" s="14" t="inlineStr">
@@ -16700,7 +16700,7 @@
       </c>
       <c r="B158" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C158" s="14" t="inlineStr">
@@ -16721,7 +16721,7 @@
       </c>
       <c r="B159" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C159" s="14" t="inlineStr">
@@ -16742,7 +16742,7 @@
       </c>
       <c r="B160" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C160" s="14" t="inlineStr">
@@ -16763,7 +16763,7 @@
       </c>
       <c r="B161" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/30 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C161" s="14" t="inlineStr">
@@ -16784,7 +16784,7 @@
       </c>
       <c r="B162" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/45 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C162" s="14" t="inlineStr">
@@ -16805,7 +16805,7 @@
       </c>
       <c r="B163" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/72 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C163" s="14" t="inlineStr">
@@ -16826,7 +16826,7 @@
       </c>
       <c r="B164" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/4.9 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C164" s="14" t="inlineStr">
@@ -16847,7 +16847,7 @@
       </c>
       <c r="B165" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-ALUM/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C165" s="14" t="inlineStr">
@@ -16868,7 +16868,7 @@
       </c>
       <c r="B166" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-ALUM/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C166" s="14" t="inlineStr">
@@ -16889,7 +16889,7 @@
       </c>
       <c r="B167" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C167" s="14" t="inlineStr">
@@ -16910,7 +16910,7 @@
       </c>
       <c r="B168" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/3.2 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C168" s="14" t="inlineStr">
@@ -16931,7 +16931,7 @@
       </c>
       <c r="B169" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/400 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C169" s="14" t="inlineStr">
@@ -16952,7 +16952,7 @@
       </c>
       <c r="B170" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C170" s="14" t="inlineStr">
@@ -16973,7 +16973,7 @@
       </c>
       <c r="B171" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C171" s="14" t="inlineStr">
@@ -16994,7 +16994,7 @@
       </c>
       <c r="B172" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/17.9 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C172" s="14" t="inlineStr">
@@ -17015,7 +17015,7 @@
       </c>
       <c r="B173" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C173" s="14" t="inlineStr">
@@ -17036,7 +17036,7 @@
       </c>
       <c r="B174" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C174" s="14" t="inlineStr">
@@ -17057,7 +17057,7 @@
       </c>
       <c r="B175" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C175" s="14" t="inlineStr">
@@ -17078,7 +17078,7 @@
       </c>
       <c r="B176" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/57 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C176" s="14" t="inlineStr">
@@ -17099,7 +17099,7 @@
       </c>
       <c r="B177" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C177" s="14" t="inlineStr">
@@ -17120,7 +17120,7 @@
       </c>
       <c r="B178" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/108 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C178" s="14" t="inlineStr">
@@ -17141,7 +17141,7 @@
       </c>
       <c r="B179" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/152 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C179" s="14" t="inlineStr">
@@ -17162,7 +17162,7 @@
       </c>
       <c r="B180" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C180" s="14" t="inlineStr">
@@ -17183,7 +17183,7 @@
       </c>
       <c r="B181" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C181" s="14" t="inlineStr">
@@ -17204,7 +17204,7 @@
       </c>
       <c r="B182" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C182" s="14" t="inlineStr">
@@ -17225,7 +17225,7 @@
       </c>
       <c r="B183" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C183" s="14" t="inlineStr">
@@ -17246,7 +17246,7 @@
       </c>
       <c r="B184" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-RL/330 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C184" s="14" t="inlineStr">
@@ -17267,7 +17267,7 @@
       </c>
       <c r="B185" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-Black/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C185" s="14" t="inlineStr">
@@ -17288,7 +17288,7 @@
       </c>
       <c r="B186" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/55 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C186" s="14" t="inlineStr">
@@ -17309,7 +17309,7 @@
       </c>
       <c r="B187" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C187" s="14" t="inlineStr">
@@ -17330,7 +17330,7 @@
       </c>
       <c r="B188" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/9.52 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C188" s="14" t="inlineStr">
@@ -17351,7 +17351,7 @@
       </c>
       <c r="B189" s="13" t="inlineStr">
         <is>
-          <t>PIT2SD/38.1 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C189" s="14" t="inlineStr">
@@ -17372,7 +17372,7 @@
       </c>
       <c r="B190" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-Black/304.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C190" s="14" t="inlineStr">
@@ -17393,7 +17393,7 @@
       </c>
       <c r="B191" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-UT/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C191" s="14" t="inlineStr">
@@ -17414,7 +17414,7 @@
       </c>
       <c r="B192" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-UT/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C192" s="14" t="inlineStr">
@@ -17435,7 +17435,7 @@
       </c>
       <c r="B193" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-UT/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C193" s="14" t="inlineStr">
@@ -17456,7 +17456,7 @@
       </c>
       <c r="B194" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-UT/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C194" s="14" t="inlineStr">
@@ -17477,7 +17477,7 @@
       </c>
       <c r="B195" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-UT/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C195" s="14" t="inlineStr">
@@ -17498,7 +17498,7 @@
       </c>
       <c r="B196" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-UT/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C196" s="14" t="inlineStr">
@@ -17519,7 +17519,7 @@
       </c>
       <c r="B197" s="13" t="inlineStr">
         <is>
-          <t>PIT3N/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C197" s="14" t="inlineStr">
@@ -17540,7 +17540,7 @@
       </c>
       <c r="B198" s="13" t="inlineStr">
         <is>
-          <t>PIT3N/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C198" s="14" t="inlineStr">
@@ -17561,7 +17561,7 @@
       </c>
       <c r="B199" s="13" t="inlineStr">
         <is>
-          <t>PIT3N/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C199" s="14" t="inlineStr">
@@ -17582,7 +17582,7 @@
       </c>
       <c r="B200" s="13" t="inlineStr">
         <is>
-          <t>PIT1AD-2RL/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C200" s="14" t="inlineStr">
@@ -17603,7 +17603,7 @@
       </c>
       <c r="B201" s="13" t="inlineStr">
         <is>
-          <t>PIT1AD-2RL/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C201" s="14" t="inlineStr">
@@ -17624,7 +17624,7 @@
       </c>
       <c r="B202" s="13" t="inlineStr">
         <is>
-          <t>PIT1AD-2RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C202" s="14" t="inlineStr">
@@ -17645,7 +17645,7 @@
       </c>
       <c r="B203" s="13" t="inlineStr">
         <is>
-          <t>PIT1AD-2RL/101.6 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C203" s="14" t="inlineStr">
@@ -17666,7 +17666,7 @@
       </c>
       <c r="B204" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/300 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C204" s="14" t="inlineStr">
@@ -17687,7 +17687,7 @@
       </c>
       <c r="B205" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-ALUM/152.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C205" s="14" t="inlineStr">
@@ -17708,7 +17708,7 @@
       </c>
       <c r="B206" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-2RL/305 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C206" s="14" t="inlineStr">
@@ -17729,7 +17729,7 @@
       </c>
       <c r="B207" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C207" s="14" t="inlineStr">
@@ -17750,7 +17750,7 @@
       </c>
       <c r="B208" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/305 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C208" s="14" t="inlineStr">
@@ -17771,7 +17771,7 @@
       </c>
       <c r="B209" s="13" t="inlineStr">
         <is>
-          <t>PIT2SD/60 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C209" s="14" t="inlineStr">
@@ -17792,7 +17792,7 @@
       </c>
       <c r="B210" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-FR/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C210" s="14" t="inlineStr">
@@ -17813,7 +17813,7 @@
       </c>
       <c r="B211" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-FR/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C211" s="14" t="inlineStr">
@@ -17834,7 +17834,7 @@
       </c>
       <c r="B212" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-FR/19 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C212" s="14" t="inlineStr">
@@ -17855,7 +17855,7 @@
       </c>
       <c r="B213" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-FR/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C213" s="14" t="inlineStr">
@@ -17876,7 +17876,7 @@
       </c>
       <c r="B214" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-FR/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C214" s="14" t="inlineStr">
@@ -17897,7 +17897,7 @@
       </c>
       <c r="B215" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/37 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C215" s="14" t="inlineStr">
@@ -17918,7 +17918,7 @@
       </c>
       <c r="B216" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-Black/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C216" s="14" t="inlineStr">
@@ -17939,7 +17939,7 @@
       </c>
       <c r="B217" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-Black/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C217" s="14" t="inlineStr">
@@ -17960,7 +17960,7 @@
       </c>
       <c r="B218" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-FR/5.08 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C218" s="14" t="inlineStr">
@@ -17981,7 +17981,7 @@
       </c>
       <c r="B219" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-ALUM/10 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C219" s="14" t="inlineStr">
@@ -18002,7 +18002,7 @@
       </c>
       <c r="B220" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-ALUM/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C220" s="14" t="inlineStr">
@@ -18023,7 +18023,7 @@
       </c>
       <c r="B221" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/9.5 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C221" s="14" t="inlineStr">
@@ -18044,7 +18044,7 @@
       </c>
       <c r="B222" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-RL/305 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C222" s="14" t="inlineStr">
@@ -18065,7 +18065,7 @@
       </c>
       <c r="B223" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-FEP616/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C223" s="14" t="inlineStr">
@@ -18086,7 +18086,7 @@
       </c>
       <c r="B224" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-FEP019/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C224" s="14" t="inlineStr">
@@ -18107,7 +18107,7 @@
       </c>
       <c r="B225" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-FEP919/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C225" s="14" t="inlineStr">
@@ -18128,7 +18128,7 @@
       </c>
       <c r="B226" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/3.17 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C226" s="14" t="inlineStr">
@@ -18149,7 +18149,7 @@
       </c>
       <c r="B227" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/3.97 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C227" s="14" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="B228" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/4.76 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C228" s="14" t="inlineStr">
@@ -18191,7 +18191,7 @@
       </c>
       <c r="B229" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/380 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C229" s="14" t="inlineStr">
@@ -18212,7 +18212,7 @@
       </c>
       <c r="B230" s="13" t="inlineStr">
         <is>
-          <t>PIT5N/159 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C230" s="14" t="inlineStr">
@@ -18233,7 +18233,7 @@
       </c>
       <c r="B231" s="13" t="inlineStr">
         <is>
-          <t>PIT1SD-2RL/76.2 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C231" s="14" t="inlineStr">
@@ -18254,7 +18254,7 @@
       </c>
       <c r="B232" s="13" t="inlineStr">
         <is>
-          <t>PET1A-Yellow/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C232" s="14" t="inlineStr">
@@ -18275,7 +18275,7 @@
       </c>
       <c r="B233" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/70 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C233" s="14" t="inlineStr">
@@ -18296,7 +18296,7 @@
       </c>
       <c r="B234" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S/70 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C234" s="14" t="inlineStr">
@@ -18317,7 +18317,7 @@
       </c>
       <c r="B235" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/70 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C235" s="14" t="inlineStr">
@@ -18338,7 +18338,7 @@
       </c>
       <c r="B236" s="13" t="inlineStr">
         <is>
-          <t>PIT2AD/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C236" s="14" t="inlineStr">
@@ -18359,7 +18359,7 @@
       </c>
       <c r="B237" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD/3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C237" s="14" t="inlineStr">
@@ -18380,7 +18380,7 @@
       </c>
       <c r="B238" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD/75 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C238" s="14" t="inlineStr">
@@ -18401,7 +18401,7 @@
       </c>
       <c r="B239" s="13" t="inlineStr">
         <is>
-          <t>PIT3N/38.1 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C239" s="14" t="inlineStr">
@@ -18422,7 +18422,7 @@
       </c>
       <c r="B240" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/7.5 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C240" s="14" t="inlineStr">
@@ -18443,7 +18443,7 @@
       </c>
       <c r="B241" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-DCD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C241" s="14" t="inlineStr">
@@ -18464,7 +18464,7 @@
       </c>
       <c r="B242" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-DCD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C242" s="14" t="inlineStr">
@@ -18485,7 +18485,7 @@
       </c>
       <c r="B243" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD-DCD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C243" s="14" t="inlineStr">
@@ -18506,7 +18506,7 @@
       </c>
       <c r="B244" s="13" t="inlineStr">
         <is>
-          <t>PIT5S-DCD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C244" s="14" t="inlineStr">
@@ -18527,7 +18527,7 @@
       </c>
       <c r="B245" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/210 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C245" s="14" t="inlineStr">
@@ -18548,7 +18548,7 @@
       </c>
       <c r="B246" s="13" t="inlineStr">
         <is>
-          <t>PET1S-Clear/8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C246" s="14" t="inlineStr">
@@ -18569,7 +18569,7 @@
       </c>
       <c r="B247" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/3.2 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C247" s="14" t="inlineStr">
@@ -18590,7 +18590,7 @@
       </c>
       <c r="B248" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/36.5 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C248" s="14" t="inlineStr">
@@ -18611,7 +18611,7 @@
       </c>
       <c r="B249" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/36.5 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C249" s="14" t="inlineStr">
@@ -18632,7 +18632,7 @@
       </c>
       <c r="B250" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/20.3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C250" s="14" t="inlineStr">
@@ -18653,7 +18653,7 @@
       </c>
       <c r="B251" s="13" t="inlineStr">
         <is>
-          <t>PET1S-Blue-DCD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C251" s="14" t="inlineStr">
@@ -18674,7 +18674,7 @@
       </c>
       <c r="B252" s="13" t="inlineStr">
         <is>
-          <t>PET2S-Blue-DCD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C252" s="14" t="inlineStr">
@@ -18695,7 +18695,7 @@
       </c>
       <c r="B253" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/7.94 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C253" s="14" t="inlineStr">
@@ -18716,7 +18716,7 @@
       </c>
       <c r="B254" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-RL/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C254" s="14" t="inlineStr">
@@ -18737,7 +18737,7 @@
       </c>
       <c r="B255" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C255" s="14" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="B256" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/254 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C256" s="14" t="inlineStr">
@@ -18779,7 +18779,7 @@
       </c>
       <c r="B257" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/22 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C257" s="14" t="inlineStr">
@@ -18800,7 +18800,7 @@
       </c>
       <c r="B258" s="13" t="inlineStr">
         <is>
-          <t>PIT5S/22 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C258" s="14" t="inlineStr">
@@ -18821,7 +18821,7 @@
       </c>
       <c r="B259" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/150 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C259" s="14" t="inlineStr">
@@ -18842,7 +18842,7 @@
       </c>
       <c r="B260" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/300 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C260" s="14" t="inlineStr">
@@ -18863,7 +18863,7 @@
       </c>
       <c r="B261" s="13" t="inlineStr">
         <is>
-          <t>PIT1S/450 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C261" s="14" t="inlineStr">
@@ -18884,7 +18884,7 @@
       </c>
       <c r="B262" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-DCD/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C262" s="14" t="inlineStr">
@@ -18905,7 +18905,7 @@
       </c>
       <c r="B263" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/230 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C263" s="14" t="inlineStr">
@@ -18926,7 +18926,7 @@
       </c>
       <c r="B264" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/50 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C264" s="14" t="inlineStr">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="B265" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/81.3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C265" s="14" t="inlineStr">
@@ -18968,7 +18968,7 @@
       </c>
       <c r="B266" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/112 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C266" s="14" t="inlineStr">
@@ -18989,7 +18989,7 @@
       </c>
       <c r="B267" s="13" t="inlineStr">
         <is>
-          <t>PIT2N/210 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C267" s="14" t="inlineStr">
@@ -19010,7 +19010,7 @@
       </c>
       <c r="B268" s="13" t="inlineStr">
         <is>
-          <t>PIT3N/210 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C268" s="14" t="inlineStr">
@@ -19031,7 +19031,7 @@
       </c>
       <c r="B269" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/9.12 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C269" s="14" t="inlineStr">
@@ -19052,7 +19052,7 @@
       </c>
       <c r="B270" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/6.73 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C270" s="14" t="inlineStr">
@@ -19073,7 +19073,7 @@
       </c>
       <c r="B271" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-Black/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C271" s="14" t="inlineStr">
@@ -19094,7 +19094,7 @@
       </c>
       <c r="B272" s="13" t="inlineStr">
         <is>
-          <t>PIT1N-ALUM/300 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C272" s="14" t="inlineStr">
@@ -19115,7 +19115,7 @@
       </c>
       <c r="B273" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-DCD/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C273" s="14" t="inlineStr">
@@ -19136,7 +19136,7 @@
       </c>
       <c r="B274" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C274" s="14" t="inlineStr">
@@ -19157,7 +19157,7 @@
       </c>
       <c r="B275" s="13" t="inlineStr">
         <is>
-          <t>PIT5N-DCD/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C275" s="14" t="inlineStr">
@@ -19178,7 +19178,7 @@
       </c>
       <c r="B276" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/30 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C276" s="14" t="inlineStr">
@@ -19199,7 +19199,7 @@
       </c>
       <c r="B277" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/40 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C277" s="14" t="inlineStr">
@@ -19220,7 +19220,7 @@
       </c>
       <c r="B278" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/60 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C278" s="14" t="inlineStr">
@@ -19241,7 +19241,7 @@
       </c>
       <c r="B279" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5SD-UT-RL/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C279" s="14" t="inlineStr">
@@ -19262,7 +19262,7 @@
       </c>
       <c r="B280" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5SD-UT-RL/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C280" s="14" t="inlineStr">
@@ -19283,7 +19283,7 @@
       </c>
       <c r="B281" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5SD-UT-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C281" s="14" t="inlineStr">
@@ -19304,7 +19304,7 @@
       </c>
       <c r="B282" s="13" t="inlineStr">
         <is>
-          <t>PIT2AD/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C282" s="14" t="inlineStr">
@@ -19325,7 +19325,7 @@
       </c>
       <c r="B283" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/15 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C283" s="14" t="inlineStr">
@@ -19346,7 +19346,7 @@
       </c>
       <c r="B284" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C284" s="14" t="inlineStr">
@@ -19367,7 +19367,7 @@
       </c>
       <c r="B285" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/116 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C285" s="14" t="inlineStr">
@@ -19388,7 +19388,7 @@
       </c>
       <c r="B286" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-T-RL/254 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C286" s="14" t="inlineStr">
@@ -19409,7 +19409,7 @@
       </c>
       <c r="B287" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-T-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C287" s="14" t="inlineStr">
@@ -19430,7 +19430,7 @@
       </c>
       <c r="B288" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-T-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C288" s="14" t="inlineStr">
@@ -19451,7 +19451,7 @@
       </c>
       <c r="B289" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5N/4.76 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C289" s="14" t="inlineStr">
@@ -19472,7 +19472,7 @@
       </c>
       <c r="B290" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C290" s="14" t="inlineStr">
@@ -19493,7 +19493,7 @@
       </c>
       <c r="B291" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-UT-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C291" s="14" t="inlineStr">
@@ -19514,7 +19514,7 @@
       </c>
       <c r="B292" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-UT-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C292" s="14" t="inlineStr">
@@ -19535,7 +19535,7 @@
       </c>
       <c r="B293" s="13" t="inlineStr">
         <is>
-          <t>PIT2AD/350 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C293" s="14" t="inlineStr">
@@ -19556,7 +19556,7 @@
       </c>
       <c r="B294" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/10 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C294" s="14" t="inlineStr">
@@ -19577,7 +19577,7 @@
       </c>
       <c r="B295" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/20 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C295" s="14" t="inlineStr">
@@ -19598,7 +19598,7 @@
       </c>
       <c r="B296" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/30 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C296" s="14" t="inlineStr">
@@ -19619,7 +19619,7 @@
       </c>
       <c r="B297" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD/6.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C297" s="14" t="inlineStr">
@@ -19640,7 +19640,7 @@
       </c>
       <c r="B298" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/9.52 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C298" s="14" t="inlineStr">
@@ -19661,7 +19661,7 @@
       </c>
       <c r="B299" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/11.11 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C299" s="14" t="inlineStr">
@@ -19682,7 +19682,7 @@
       </c>
       <c r="B300" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ALUM/254 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C300" s="14" t="inlineStr">
@@ -19703,7 +19703,7 @@
       </c>
       <c r="B301" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5SD-UT-RL/112 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C301" s="14" t="inlineStr">
@@ -19724,7 +19724,7 @@
       </c>
       <c r="B302" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5SD-UT-RL/284 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C302" s="14" t="inlineStr">
@@ -19745,7 +19745,7 @@
       </c>
       <c r="B303" s="13" t="inlineStr">
         <is>
-          <t>PIT3N/152.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C303" s="14" t="inlineStr">
@@ -19766,7 +19766,7 @@
       </c>
       <c r="B304" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/5 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C304" s="14" t="inlineStr">
@@ -19787,7 +19787,7 @@
       </c>
       <c r="B305" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-T-RL/44 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C305" s="14" t="inlineStr">
@@ -19808,7 +19808,7 @@
       </c>
       <c r="B306" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-LO/355 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C306" s="14" t="inlineStr">
@@ -19829,7 +19829,7 @@
       </c>
       <c r="B307" s="13" t="inlineStr">
         <is>
-          <t>PIT3S/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C307" s="14" t="inlineStr">
@@ -19850,7 +19850,7 @@
       </c>
       <c r="B308" s="13" t="inlineStr">
         <is>
-          <t>PIT3S-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C308" s="14" t="inlineStr">
@@ -19871,7 +19871,7 @@
       </c>
       <c r="B309" s="13" t="inlineStr">
         <is>
-          <t>PIT3S/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C309" s="14" t="inlineStr">
@@ -19892,7 +19892,7 @@
       </c>
       <c r="B310" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C310" s="14" t="inlineStr">
@@ -19913,7 +19913,7 @@
       </c>
       <c r="B311" s="13" t="inlineStr">
         <is>
-          <t>PIT3S-RL/50 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C311" s="14" t="inlineStr">
@@ -19934,7 +19934,7 @@
       </c>
       <c r="B312" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-T-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C312" s="14" t="inlineStr">
@@ -19955,7 +19955,7 @@
       </c>
       <c r="B313" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-T-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C313" s="14" t="inlineStr">
@@ -19976,7 +19976,7 @@
       </c>
       <c r="B314" s="13" t="inlineStr">
         <is>
-          <t>PIT3S-T-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C314" s="14" t="inlineStr">
@@ -19997,7 +19997,7 @@
       </c>
       <c r="B315" s="13" t="inlineStr">
         <is>
-          <t>PIT3S-T-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C315" s="14" t="inlineStr">
@@ -20018,7 +20018,7 @@
       </c>
       <c r="B316" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-LO/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C316" s="14" t="inlineStr">
@@ -20039,7 +20039,7 @@
       </c>
       <c r="B317" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-LO/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C317" s="14" t="inlineStr">
@@ -20060,7 +20060,7 @@
       </c>
       <c r="B318" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-LO/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C318" s="14" t="inlineStr">
@@ -20081,7 +20081,7 @@
       </c>
       <c r="B319" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-LO/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C319" s="14" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="B320" s="13" t="inlineStr">
         <is>
-          <t>PIT2S2-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C320" s="14" t="inlineStr">
@@ -20123,7 +20123,7 @@
       </c>
       <c r="B321" s="13" t="inlineStr">
         <is>
-          <t>PIT2S2-RL/114 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C321" s="14" t="inlineStr">
@@ -20144,7 +20144,7 @@
       </c>
       <c r="B322" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-B/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C322" s="14" t="inlineStr">
@@ -20165,7 +20165,7 @@
       </c>
       <c r="B323" s="13" t="inlineStr">
         <is>
-          <t>PIT2S/21.5 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C323" s="14" t="inlineStr">
@@ -20186,7 +20186,7 @@
       </c>
       <c r="B324" s="13" t="inlineStr">
         <is>
-          <t>PIT2AD-LO/355 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C324" s="14" t="inlineStr">
@@ -20207,7 +20207,7 @@
       </c>
       <c r="B325" s="13" t="inlineStr">
         <is>
-          <t>PIT2AD-LO/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C325" s="14" t="inlineStr">
@@ -20228,7 +20228,7 @@
       </c>
       <c r="B326" s="13" t="inlineStr">
         <is>
-          <t>PIT2AD-LO/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C326" s="14" t="inlineStr">
@@ -20249,7 +20249,7 @@
       </c>
       <c r="B327" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-Black/152.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C327" s="14" t="inlineStr">
@@ -20270,7 +20270,7 @@
       </c>
       <c r="B328" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-BRL/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C328" s="14" t="inlineStr">
@@ -20291,7 +20291,7 @@
       </c>
       <c r="B329" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-BRL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C329" s="14" t="inlineStr">
@@ -20312,7 +20312,7 @@
       </c>
       <c r="B330" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-BRL/304.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C330" s="14" t="inlineStr">
@@ -20333,7 +20333,7 @@
       </c>
       <c r="B331" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-BRL/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C331" s="14" t="inlineStr">
@@ -20354,7 +20354,7 @@
       </c>
       <c r="B332" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD-BRL/152.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C332" s="14" t="inlineStr">
@@ -20375,7 +20375,7 @@
       </c>
       <c r="B333" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/63.5 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C333" s="14" t="inlineStr">
@@ -20396,7 +20396,7 @@
       </c>
       <c r="B334" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-T-RL/162 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C334" s="14" t="inlineStr">
@@ -20417,7 +20417,7 @@
       </c>
       <c r="B335" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-T-RL/162 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C335" s="14" t="inlineStr">
@@ -20438,7 +20438,7 @@
       </c>
       <c r="B336" s="13" t="inlineStr">
         <is>
-          <t>PIT2S-RL/162 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C336" s="14" t="inlineStr">
@@ -20459,7 +20459,7 @@
       </c>
       <c r="B337" s="13" t="inlineStr">
         <is>
-          <t>PET2S-Green/101.6 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C337" s="14" t="inlineStr">
@@ -20480,7 +20480,7 @@
       </c>
       <c r="B338" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C338" s="14" t="inlineStr">
@@ -20501,7 +20501,7 @@
       </c>
       <c r="B339" s="13" t="inlineStr">
         <is>
-          <t>PET1A-Yellow/32 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C339" s="14" t="inlineStr">
@@ -20522,7 +20522,7 @@
       </c>
       <c r="B340" s="13" t="inlineStr">
         <is>
-          <t>PET1A-Yellow/28 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C340" s="14" t="inlineStr">
@@ -20543,7 +20543,7 @@
       </c>
       <c r="B341" s="13" t="inlineStr">
         <is>
-          <t>PET1A-Yellow/26 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C341" s="14" t="inlineStr">
@@ -20564,7 +20564,7 @@
       </c>
       <c r="B342" s="13" t="inlineStr">
         <is>
-          <t>PET1A-Yellow/17 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C342" s="14" t="inlineStr">
@@ -20585,7 +20585,7 @@
       </c>
       <c r="B343" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/254 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C343" s="14" t="inlineStr">
@@ -20606,7 +20606,7 @@
       </c>
       <c r="B344" s="13" t="inlineStr">
         <is>
-          <t>PIT2A/60 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C344" s="14" t="inlineStr">
@@ -20627,7 +20627,7 @@
       </c>
       <c r="B345" s="13" t="inlineStr">
         <is>
-          <t>PET1A-Yellow/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C345" s="14" t="inlineStr">
@@ -20648,7 +20648,7 @@
       </c>
       <c r="B346" s="13" t="inlineStr">
         <is>
-          <t>PET1A-Yellow/38.1 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C346" s="14" t="inlineStr">
@@ -20669,7 +20669,7 @@
       </c>
       <c r="B347" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-T-RL/164 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C347" s="14" t="inlineStr">
@@ -20690,7 +20690,7 @@
       </c>
       <c r="B348" s="13" t="inlineStr">
         <is>
-          <t>PIT3N/14 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C348" s="14" t="inlineStr">
@@ -20711,7 +20711,7 @@
       </c>
       <c r="B349" s="13" t="inlineStr">
         <is>
-          <t>PET2S-Green/38 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C349" s="14" t="inlineStr">
@@ -20732,7 +20732,7 @@
       </c>
       <c r="B350" s="13" t="inlineStr">
         <is>
-          <t>PET2S-Green/76 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C350" s="14" t="inlineStr">
@@ -20753,7 +20753,7 @@
       </c>
       <c r="B351" s="13" t="inlineStr">
         <is>
-          <t>PIT5S-RL/12.7 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C351" s="14" t="inlineStr">
@@ -20774,7 +20774,7 @@
       </c>
       <c r="B352" s="13" t="inlineStr">
         <is>
-          <t>PIT5S-RL/25.4 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C352" s="14" t="inlineStr">
@@ -20795,7 +20795,7 @@
       </c>
       <c r="B353" s="13" t="inlineStr">
         <is>
-          <t>PIT5S-RL/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C353" s="14" t="inlineStr">
@@ -20816,7 +20816,7 @@
       </c>
       <c r="B354" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-ESD/200 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C354" s="14" t="inlineStr">
@@ -20837,7 +20837,7 @@
       </c>
       <c r="B355" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-WL-SG/12 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C355" s="14" t="inlineStr">
@@ -20858,7 +20858,7 @@
       </c>
       <c r="B356" s="13" t="inlineStr">
         <is>
-          <t>PIT1A/36.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C356" s="14" t="inlineStr">
@@ -20879,7 +20879,7 @@
       </c>
       <c r="B357" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-FRC/12 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C357" s="14" t="inlineStr">
@@ -20900,7 +20900,7 @@
       </c>
       <c r="B358" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL/70 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C358" s="14" t="inlineStr">
@@ -20921,7 +20921,7 @@
       </c>
       <c r="B359" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-UT/38.1 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C359" s="14" t="inlineStr">
@@ -20942,7 +20942,7 @@
       </c>
       <c r="B360" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-UT-RL/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C360" s="14" t="inlineStr">
@@ -20963,7 +20963,7 @@
       </c>
       <c r="B361" s="13" t="inlineStr">
         <is>
-          <t>PET1S-Clear/38.1 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C361" s="14" t="inlineStr">
@@ -20984,7 +20984,7 @@
       </c>
       <c r="B362" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-B/50.8 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C362" s="14" t="inlineStr">
@@ -21005,7 +21005,7 @@
       </c>
       <c r="B363" s="13" t="inlineStr">
         <is>
-          <t>PET1S-UT-Clear/38.1 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C363" s="14" t="inlineStr">
@@ -21026,7 +21026,7 @@
       </c>
       <c r="B364" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT/200 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C364" s="14" t="inlineStr">
@@ -21047,7 +21047,7 @@
       </c>
       <c r="B365" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-T-RL/62 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C365" s="14" t="inlineStr">
@@ -21068,7 +21068,7 @@
       </c>
       <c r="B366" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-UT-RL/62 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C366" s="14" t="inlineStr">
@@ -21089,7 +21089,7 @@
       </c>
       <c r="B367" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-WL-SG/100 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C367" s="14" t="inlineStr">
@@ -21110,7 +21110,7 @@
       </c>
       <c r="B368" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-LO/400 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C368" s="14" t="inlineStr">
@@ -21131,7 +21131,7 @@
       </c>
       <c r="B369" s="13" t="inlineStr">
         <is>
-          <t>PIT1A-LO/400 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C369" s="14" t="inlineStr">
@@ -21152,7 +21152,7 @@
       </c>
       <c r="B370" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/4.3 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C370" s="14" t="inlineStr">
@@ -21173,7 +21173,7 @@
       </c>
       <c r="B371" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/160 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C371" s="14" t="inlineStr">
@@ -21194,7 +21194,7 @@
       </c>
       <c r="B372" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/200 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C372" s="14" t="inlineStr">
@@ -21215,7 +21215,7 @@
       </c>
       <c r="B373" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-B/190 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C373" s="14" t="inlineStr">
@@ -21236,7 +21236,7 @@
       </c>
       <c r="B374" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL-Series/64.45 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C374" s="14" t="inlineStr">
@@ -21257,7 +21257,7 @@
       </c>
       <c r="B375" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-RL-Series/54.35 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C375" s="14" t="inlineStr">
@@ -21278,7 +21278,7 @@
       </c>
       <c r="B376" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-ESD-Series/330 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C376" s="14" t="inlineStr">
@@ -21299,7 +21299,7 @@
       </c>
       <c r="B377" s="13" t="inlineStr">
         <is>
-          <t>PIT2A-FR Series/65 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C377" s="14" t="inlineStr">
@@ -21320,7 +21320,7 @@
       </c>
       <c r="B378" s="13" t="inlineStr">
         <is>
-          <t>PIT0.5S-UT-RL/164 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C378" s="14" t="inlineStr">
@@ -21341,7 +21341,7 @@
       </c>
       <c r="B379" s="13" t="inlineStr">
         <is>
-          <t>PIT1S-UT-RL/164 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C379" s="14" t="inlineStr">
@@ -21362,7 +21362,7 @@
       </c>
       <c r="B380" s="13" t="inlineStr">
         <is>
-          <t>PIT1N/164 Rev 1</t>
+          <t>Rev 1</t>
         </is>
       </c>
       <c r="C380" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Make outsourcing charge component names revision specific
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R4gmyWjX7HwofLtwBHfu93
</commit_message>
<xml_diff>
--- a/Krayden_Europe_-_Bill_of_Materials_Transformed.xlsx
+++ b/Krayden_Europe_-_Bill_of_Materials_Transformed.xlsx
@@ -21400,7 +21400,7 @@
     <col width="9.140625" customWidth="1" style="5" min="7" max="8"/>
     <col width="18" bestFit="1" customWidth="1" style="5" min="9" max="9"/>
     <col width="53" bestFit="1" customWidth="1" style="5" min="10" max="10"/>
-    <col width="9.140625" customWidth="1" style="5" min="11" max="16384"/>
+    <col width="60" customWidth="1" style="5" min="11" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -21454,6 +21454,11 @@
           <t>MPN</t>
         </is>
       </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Review Flag</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -21576,7 +21581,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>GDL2200 | 113mm Circle</t>
         </is>
       </c>
       <c r="C6" s="15" t="n"/>
@@ -21623,7 +21628,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>GDL2900 | 58mm Circle</t>
         </is>
       </c>
       <c r="C8" s="14" t="n"/>
@@ -21670,7 +21675,7 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>GDL1500 | 113mm Circle</t>
         </is>
       </c>
       <c r="C10" s="14" t="n"/>
@@ -21717,7 +21722,7 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>GDL1500 | 60x60mm sheet 4x R6 corners</t>
         </is>
       </c>
       <c r="C12" s="14" t="n"/>
@@ -21766,7 +21771,7 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>GDL1850 | 400 x 400mm Sheet</t>
         </is>
       </c>
       <c r="C14" s="14" t="n"/>
@@ -21815,7 +21820,7 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>MREC909 | 275gr can</t>
         </is>
       </c>
       <c r="C16" s="14" t="n"/>
@@ -21862,7 +21867,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.350mm (14mil)</t>
         </is>
       </c>
       <c r="C18" s="14" t="n"/>
@@ -21909,7 +21914,7 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR7 | 0.457mm (18mil)</t>
         </is>
       </c>
       <c r="C20" s="14" t="n"/>
@@ -21956,7 +21961,7 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.457mm (18mil)</t>
         </is>
       </c>
       <c r="C22" s="14" t="n"/>
@@ -22003,7 +22008,7 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.300mm (12mil)</t>
         </is>
       </c>
       <c r="C24" s="14" t="n"/>
@@ -22050,7 +22055,7 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.250mm (10mil)</t>
         </is>
       </c>
       <c r="C26" s="14" t="n"/>
@@ -22097,7 +22102,7 @@
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.350mm (14mil)</t>
         </is>
       </c>
       <c r="C28" s="14" t="n"/>
@@ -22144,7 +22149,7 @@
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-Sn63Pb37 | 0.560mm (22mil)</t>
         </is>
       </c>
       <c r="C30" s="14" t="n"/>
@@ -22191,7 +22196,7 @@
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR7 | 0.300mm (11.8mil)</t>
         </is>
       </c>
       <c r="C32" s="14" t="n"/>
@@ -22238,7 +22243,7 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.500mm (19.6mil)</t>
         </is>
       </c>
       <c r="C34" s="14" t="n"/>
@@ -22285,7 +22290,7 @@
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR7 | 0.500mm (19.6mil)</t>
         </is>
       </c>
       <c r="C36" s="14" t="n"/>
@@ -22332,7 +22337,7 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR7-Bi58Sn42 | 0.300mm (11.8mil)</t>
         </is>
       </c>
       <c r="C38" s="14" t="n"/>
@@ -22379,7 +22384,7 @@
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR7-Bi58Sn42 | 0.500mm (19.6mil)</t>
         </is>
       </c>
       <c r="C40" s="14" t="n"/>
@@ -22426,7 +22431,7 @@
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-Bi58Sn42 | 0.300mm (12mil)</t>
         </is>
       </c>
       <c r="C42" s="14" t="n"/>
@@ -22473,7 +22478,7 @@
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-Bi58Sn42 | 0.500mm (19.6mil)</t>
         </is>
       </c>
       <c r="C44" s="14" t="n"/>
@@ -22520,7 +22525,7 @@
       </c>
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR7 | 0.400mm (15.7mil)</t>
         </is>
       </c>
       <c r="C46" s="14" t="n"/>
@@ -22567,7 +22572,7 @@
       </c>
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.400mm (15.7mil)</t>
         </is>
       </c>
       <c r="C48" s="14" t="n"/>
@@ -22614,7 +22619,7 @@
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC105 | 0.300mm (12mil)</t>
         </is>
       </c>
       <c r="C50" s="14" t="n"/>
@@ -22661,7 +22666,7 @@
       </c>
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-CCSAC305 | 0.350mm (14mil)</t>
         </is>
       </c>
       <c r="C52" s="14" t="n"/>
@@ -22708,7 +22713,7 @@
       </c>
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-Sn10Pb90 | 0.380mm (15mil)</t>
         </is>
       </c>
       <c r="C54" s="14" t="n"/>
@@ -22755,7 +22760,7 @@
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-Sn10Pb90 | 0.500mm (15mil)</t>
         </is>
       </c>
       <c r="C56" s="14" t="n"/>
@@ -22802,7 +22807,7 @@
       </c>
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.600mm (23.6mil)</t>
         </is>
       </c>
       <c r="C58" s="14" t="n"/>
@@ -22849,7 +22854,7 @@
       </c>
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>TR13-SAC305 | 0.760mm (30mil)</t>
         </is>
       </c>
       <c r="C60" s="14" t="n"/>
@@ -22896,7 +22901,7 @@
       </c>
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 3mm (0.118") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C62" s="14" t="n"/>
@@ -22943,7 +22948,7 @@
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 12mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C64" s="14" t="n"/>
@@ -22990,7 +22995,7 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C66" s="14" t="n"/>
@@ -23037,7 +23042,7 @@
       </c>
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C68" s="14" t="n"/>
@@ -23084,7 +23089,7 @@
       </c>
       <c r="B70" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C70" s="14" t="n"/>
@@ -23131,7 +23136,7 @@
       </c>
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 20mm (0.79") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C72" s="14" t="n"/>
@@ -23178,7 +23183,7 @@
       </c>
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 25mm (0.98") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C74" s="14" t="n"/>
@@ -23225,7 +23230,7 @@
       </c>
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C76" s="14" t="n"/>
@@ -23272,7 +23277,7 @@
       </c>
       <c r="B78" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C78" s="14" t="n"/>
@@ -23336,6 +23341,11 @@
           <t>Outsourcing Charge</t>
         </is>
       </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>No product report match for PIT1A/101 - name not updated</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="14" t="inlineStr">
@@ -23366,7 +23376,7 @@
       </c>
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 3mm (0.118") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C82" s="14" t="n"/>
@@ -23413,7 +23423,7 @@
       </c>
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C84" s="14" t="n"/>
@@ -23460,7 +23470,7 @@
       </c>
       <c r="B86" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 12mm (0.47") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C86" s="14" t="n"/>
@@ -23507,7 +23517,7 @@
       </c>
       <c r="B88" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C88" s="14" t="n"/>
@@ -23554,7 +23564,7 @@
       </c>
       <c r="B90" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C90" s="14" t="n"/>
@@ -23601,7 +23611,7 @@
       </c>
       <c r="B92" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 20mm (0.79") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C92" s="14" t="n"/>
@@ -23648,7 +23658,7 @@
       </c>
       <c r="B94" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 25mm (0.98") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C94" s="14" t="n"/>
@@ -23695,7 +23705,7 @@
       </c>
       <c r="B96" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C96" s="14" t="n"/>
@@ -23742,7 +23752,7 @@
       </c>
       <c r="B98" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C98" s="14" t="n"/>
@@ -23789,7 +23799,7 @@
       </c>
       <c r="B100" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C100" s="14" t="n"/>
@@ -23836,7 +23846,7 @@
       </c>
       <c r="B102" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 200mm (7.9") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C102" s="14" t="n"/>
@@ -23883,7 +23893,7 @@
       </c>
       <c r="B104" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 3mm (0.118") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C104" s="14" t="n"/>
@@ -23930,7 +23940,7 @@
       </c>
       <c r="B106" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C106" s="14" t="n"/>
@@ -23977,7 +23987,7 @@
       </c>
       <c r="B108" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 12mm (0.47") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C108" s="14" t="n"/>
@@ -24024,7 +24034,7 @@
       </c>
       <c r="B110" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C110" s="14" t="n"/>
@@ -24071,7 +24081,7 @@
       </c>
       <c r="B112" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C112" s="14" t="n"/>
@@ -24118,7 +24128,7 @@
       </c>
       <c r="B114" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 20mm (0.79") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C114" s="14" t="n"/>
@@ -24165,7 +24175,7 @@
       </c>
       <c r="B116" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 25mm (0.98") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C116" s="14" t="n"/>
@@ -24212,7 +24222,7 @@
       </c>
       <c r="B118" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C118" s="14" t="n"/>
@@ -24259,7 +24269,7 @@
       </c>
       <c r="B120" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C120" s="14" t="n"/>
@@ -24306,7 +24316,7 @@
       </c>
       <c r="B122" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C122" s="14" t="n"/>
@@ -24353,7 +24363,7 @@
       </c>
       <c r="B124" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 3mm (0.118") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C124" s="14" t="n"/>
@@ -24400,7 +24410,7 @@
       </c>
       <c r="B126" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C126" s="14" t="n"/>
@@ -24447,7 +24457,7 @@
       </c>
       <c r="B128" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 12mm (0.47") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C128" s="14" t="n"/>
@@ -24494,7 +24504,7 @@
       </c>
       <c r="B130" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C130" s="14" t="n"/>
@@ -24541,7 +24551,7 @@
       </c>
       <c r="B132" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C132" s="14" t="n"/>
@@ -24588,7 +24598,7 @@
       </c>
       <c r="B134" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 20mm (0.79") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C134" s="14" t="n"/>
@@ -24635,7 +24645,7 @@
       </c>
       <c r="B136" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 25mm (0.98") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C136" s="14" t="n"/>
@@ -24682,7 +24692,7 @@
       </c>
       <c r="B138" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C138" s="14" t="n"/>
@@ -24729,7 +24739,7 @@
       </c>
       <c r="B140" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C140" s="14" t="n"/>
@@ -24776,7 +24786,7 @@
       </c>
       <c r="B142" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C142" s="14" t="n"/>
@@ -24823,7 +24833,7 @@
       </c>
       <c r="B144" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2SD | 6.4mm (¼") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C144" s="14" t="n"/>
@@ -24870,7 +24880,7 @@
       </c>
       <c r="B146" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2SD | 12.7mm (½") wide x 33m (36 yd) long</t>
         </is>
       </c>
       <c r="C146" s="14" t="n"/>
@@ -24917,7 +24927,7 @@
       </c>
       <c r="B148" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2SD | 19mm (¾") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C148" s="14" t="n"/>
@@ -24964,7 +24974,7 @@
       </c>
       <c r="B150" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2SD | 25.4mm (1") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C150" s="14" t="n"/>
@@ -25011,7 +25021,7 @@
       </c>
       <c r="B152" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2SD | 50.8mm (2") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C152" s="14" t="n"/>
@@ -25058,7 +25068,7 @@
       </c>
       <c r="B154" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C154" s="14" t="n"/>
@@ -25105,7 +25115,7 @@
       </c>
       <c r="B156" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C156" s="14" t="n"/>
@@ -25152,7 +25162,7 @@
       </c>
       <c r="B158" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C158" s="14" t="n"/>
@@ -25199,7 +25209,7 @@
       </c>
       <c r="B160" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C160" s="14" t="n"/>
@@ -25246,7 +25256,7 @@
       </c>
       <c r="B162" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C162" s="14" t="n"/>
@@ -25293,7 +25303,7 @@
       </c>
       <c r="B164" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-WL-SG | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C164" s="14" t="n"/>
@@ -25340,7 +25350,7 @@
       </c>
       <c r="B166" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-WL-SG | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C166" s="14" t="n"/>
@@ -25387,7 +25397,7 @@
       </c>
       <c r="B168" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-WL-SG | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C168" s="14" t="n"/>
@@ -25434,7 +25444,7 @@
       </c>
       <c r="B170" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-WL-SG | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C170" s="14" t="n"/>
@@ -25481,7 +25491,7 @@
       </c>
       <c r="B172" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-WL-SG | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C172" s="14" t="n"/>
@@ -25528,7 +25538,7 @@
       </c>
       <c r="B174" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-Blue | 6.4mm (¼") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C174" s="14" t="n"/>
@@ -25575,7 +25585,7 @@
       </c>
       <c r="B176" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-Blue | 12.7mm (½") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C176" s="14" t="n"/>
@@ -25622,7 +25632,7 @@
       </c>
       <c r="B178" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-Blue | 19mm (¾") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C178" s="14" t="n"/>
@@ -25669,7 +25679,7 @@
       </c>
       <c r="B180" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-Blue | 25.4mm (1") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C180" s="14" t="n"/>
@@ -25716,7 +25726,7 @@
       </c>
       <c r="B182" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-Blue | 50.8mm (2") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C182" s="14" t="n"/>
@@ -25763,7 +25773,7 @@
       </c>
       <c r="B184" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C184" s="14" t="n"/>
@@ -25810,7 +25820,7 @@
       </c>
       <c r="B186" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C186" s="14" t="n"/>
@@ -25857,7 +25867,7 @@
       </c>
       <c r="B188" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C188" s="14" t="n"/>
@@ -25904,7 +25914,7 @@
       </c>
       <c r="B190" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C190" s="14" t="n"/>
@@ -25951,7 +25961,7 @@
       </c>
       <c r="B192" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C192" s="14" t="n"/>
@@ -25998,7 +26008,7 @@
       </c>
       <c r="B194" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C194" s="14" t="n"/>
@@ -26045,7 +26055,7 @@
       </c>
       <c r="B196" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C196" s="14" t="n"/>
@@ -26092,7 +26102,7 @@
       </c>
       <c r="B198" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C198" s="14" t="n"/>
@@ -26139,7 +26149,7 @@
       </c>
       <c r="B200" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C200" s="14" t="n"/>
@@ -26186,7 +26196,7 @@
       </c>
       <c r="B202" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C202" s="14" t="n"/>
@@ -26233,7 +26243,7 @@
       </c>
       <c r="B204" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C204" s="14" t="n"/>
@@ -26280,7 +26290,7 @@
       </c>
       <c r="B206" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 4.2mm (0.165") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C206" s="14" t="n"/>
@@ -26327,7 +26337,7 @@
       </c>
       <c r="B208" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C208" s="14" t="n"/>
@@ -26374,7 +26384,7 @@
       </c>
       <c r="B210" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 4.2mm (0.165") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C210" s="14" t="n"/>
@@ -26421,7 +26431,7 @@
       </c>
       <c r="B212" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C212" s="14" t="n"/>
@@ -26468,7 +26478,7 @@
       </c>
       <c r="B214" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C214" s="14" t="n"/>
@@ -26515,7 +26525,7 @@
       </c>
       <c r="B216" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C216" s="14" t="n"/>
@@ -26562,7 +26572,7 @@
       </c>
       <c r="B218" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C218" s="14" t="n"/>
@@ -26609,7 +26619,7 @@
       </c>
       <c r="B220" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C220" s="14" t="n"/>
@@ -26656,7 +26666,7 @@
       </c>
       <c r="B222" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C222" s="14" t="n"/>
@@ -26703,7 +26713,7 @@
       </c>
       <c r="B224" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C224" s="14" t="n"/>
@@ -26750,7 +26760,7 @@
       </c>
       <c r="B226" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C226" s="14" t="n"/>
@@ -26797,7 +26807,7 @@
       </c>
       <c r="B228" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C228" s="14" t="n"/>
@@ -26844,7 +26854,7 @@
       </c>
       <c r="B230" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C230" s="14" t="n"/>
@@ -26891,7 +26901,7 @@
       </c>
       <c r="B232" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C232" s="14" t="n"/>
@@ -26938,7 +26948,7 @@
       </c>
       <c r="B234" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C234" s="14" t="n"/>
@@ -26985,7 +26995,7 @@
       </c>
       <c r="B236" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 150mm (5.91") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C236" s="14" t="n"/>
@@ -27032,7 +27042,7 @@
       </c>
       <c r="B238" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C238" s="14" t="n"/>
@@ -27079,7 +27089,7 @@
       </c>
       <c r="B240" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 101.6mm (4") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C240" s="14" t="n"/>
@@ -27126,7 +27136,7 @@
       </c>
       <c r="B242" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 254mm (10") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C242" s="14" t="n"/>
@@ -27173,7 +27183,7 @@
       </c>
       <c r="B244" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 304.8mm (12") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C244" s="14" t="n"/>
@@ -27220,7 +27230,7 @@
       </c>
       <c r="B246" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 203.2mm (8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C246" s="14" t="n"/>
@@ -27267,7 +27277,7 @@
       </c>
       <c r="B248" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 6.4mm (1/4") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C248" s="14" t="n"/>
@@ -27314,7 +27324,7 @@
       </c>
       <c r="B250" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 17.9mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C250" s="14" t="n"/>
@@ -27361,7 +27371,7 @@
       </c>
       <c r="B252" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C252" s="14" t="n"/>
@@ -27408,7 +27418,7 @@
       </c>
       <c r="B254" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C254" s="14" t="n"/>
@@ -27455,7 +27465,7 @@
       </c>
       <c r="B256" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C256" s="14" t="n"/>
@@ -27502,7 +27512,7 @@
       </c>
       <c r="B258" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C258" s="14" t="n"/>
@@ -27549,7 +27559,7 @@
       </c>
       <c r="B260" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C260" s="14" t="n"/>
@@ -27596,7 +27606,7 @@
       </c>
       <c r="B262" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-2RL | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C262" s="14" t="n"/>
@@ -27643,7 +27653,7 @@
       </c>
       <c r="B264" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-2RL | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C264" s="14" t="n"/>
@@ -27690,7 +27700,7 @@
       </c>
       <c r="B266" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-2RL | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C266" s="14" t="n"/>
@@ -27737,7 +27747,7 @@
       </c>
       <c r="B268" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-2RL | 101.6mm (4") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C268" s="14" t="n"/>
@@ -27784,7 +27794,7 @@
       </c>
       <c r="B270" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 180mm (7.09") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C270" s="14" t="n"/>
@@ -27831,7 +27841,7 @@
       </c>
       <c r="B272" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 101.6mm (4") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C272" s="14" t="n"/>
@@ -27878,7 +27888,7 @@
       </c>
       <c r="B274" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD | 100mm (3.94") wide x 30m (36yd) long</t>
         </is>
       </c>
       <c r="C274" s="14" t="n"/>
@@ -27925,7 +27935,7 @@
       </c>
       <c r="B276" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD | 12.7mm (½") wide x 33m (36 yd) long</t>
         </is>
       </c>
       <c r="C276" s="14" t="n"/>
@@ -27972,7 +27982,7 @@
       </c>
       <c r="B278" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD | 19mm (¾") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C278" s="14" t="n"/>
@@ -28019,7 +28029,7 @@
       </c>
       <c r="B280" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C280" s="14" t="n"/>
@@ -28066,7 +28076,7 @@
       </c>
       <c r="B282" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD | 50.8mm (2") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C282" s="14" t="n"/>
@@ -28113,7 +28123,7 @@
       </c>
       <c r="B284" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD | 6.4mm (¼") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C284" s="14" t="n"/>
@@ -28160,7 +28170,7 @@
       </c>
       <c r="B286" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N | 96.5mm (3.8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C286" s="14" t="n"/>
@@ -28207,7 +28217,7 @@
       </c>
       <c r="B288" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 40mm (1.57") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C288" s="14" t="n"/>
@@ -28254,7 +28264,7 @@
       </c>
       <c r="B290" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 127mm (5") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C290" s="14" t="n"/>
@@ -28301,7 +28311,7 @@
       </c>
       <c r="B292" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 152mm (6") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C292" s="14" t="n"/>
@@ -28348,7 +28358,7 @@
       </c>
       <c r="B294" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 27mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C294" s="14" t="n"/>
@@ -28395,7 +28405,7 @@
       </c>
       <c r="B296" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 9mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C296" s="14" t="n"/>
@@ -28442,7 +28452,7 @@
       </c>
       <c r="B298" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 93mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C298" s="14" t="n"/>
@@ -28489,7 +28499,7 @@
       </c>
       <c r="B300" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 9.53mm (3/8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C300" s="14" t="n"/>
@@ -28536,7 +28546,7 @@
       </c>
       <c r="B302" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 3mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C302" s="14" t="n"/>
@@ -28583,7 +28593,7 @@
       </c>
       <c r="B304" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C304" s="14" t="n"/>
@@ -28630,7 +28640,7 @@
       </c>
       <c r="B306" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C306" s="14" t="n"/>
@@ -28677,7 +28687,7 @@
       </c>
       <c r="B308" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C308" s="14" t="n"/>
@@ -28724,7 +28734,7 @@
       </c>
       <c r="B310" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C310" s="14" t="n"/>
@@ -28771,7 +28781,7 @@
       </c>
       <c r="B312" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 36.8mm (1.45") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C312" s="14" t="n"/>
@@ -28818,7 +28828,7 @@
       </c>
       <c r="B314" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C314" s="14" t="n"/>
@@ -28865,7 +28875,7 @@
       </c>
       <c r="B316" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C316" s="14" t="n"/>
@@ -28912,7 +28922,7 @@
       </c>
       <c r="B318" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C318" s="14" t="n"/>
@@ -28959,7 +28969,7 @@
       </c>
       <c r="B320" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 30mm (1.18") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C320" s="14" t="n"/>
@@ -29006,7 +29016,7 @@
       </c>
       <c r="B322" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 45mm (2.83") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C322" s="14" t="n"/>
@@ -29053,7 +29063,7 @@
       </c>
       <c r="B324" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 72mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C324" s="14" t="n"/>
@@ -29100,7 +29110,7 @@
       </c>
       <c r="B326" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 4.9mm (0.193") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C326" s="14" t="n"/>
@@ -29147,7 +29157,7 @@
       </c>
       <c r="B328" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-ALUM | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C328" s="14" t="n"/>
@@ -29194,7 +29204,7 @@
       </c>
       <c r="B330" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-ALUM | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C330" s="14" t="n"/>
@@ -29241,7 +29251,7 @@
       </c>
       <c r="B332" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 100mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C332" s="14" t="n"/>
@@ -29288,7 +29298,7 @@
       </c>
       <c r="B334" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 3.2mm (1/8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C334" s="14" t="n"/>
@@ -29335,7 +29345,7 @@
       </c>
       <c r="B336" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 0.5-mil Polyimide Film No Adhesive</t>
         </is>
       </c>
       <c r="C336" s="14" t="n"/>
@@ -29382,7 +29392,7 @@
       </c>
       <c r="B338" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C338" s="14" t="n"/>
@@ -29429,7 +29439,7 @@
       </c>
       <c r="B340" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C340" s="14" t="n"/>
@@ -29476,7 +29486,7 @@
       </c>
       <c r="B342" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 17.9mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C342" s="14" t="n"/>
@@ -29523,7 +29533,7 @@
       </c>
       <c r="B344" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C344" s="14" t="n"/>
@@ -29570,7 +29580,7 @@
       </c>
       <c r="B346" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C346" s="14" t="n"/>
@@ -29617,7 +29627,7 @@
       </c>
       <c r="B348" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C348" s="14" t="n"/>
@@ -29664,7 +29674,7 @@
       </c>
       <c r="B350" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 57mm (2.25") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C350" s="14" t="n"/>
@@ -29711,7 +29721,7 @@
       </c>
       <c r="B352" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C352" s="14" t="n"/>
@@ -29758,7 +29768,7 @@
       </c>
       <c r="B354" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 108mm (4.25") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C354" s="14" t="n"/>
@@ -29805,7 +29815,7 @@
       </c>
       <c r="B356" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 152mm (6") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C356" s="14" t="n"/>
@@ -29852,7 +29862,7 @@
       </c>
       <c r="B358" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD | 100mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C358" s="14" t="n"/>
@@ -29899,7 +29909,7 @@
       </c>
       <c r="B360" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD | 12.7mm (0.5 in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C360" s="14" t="n"/>
@@ -29946,7 +29956,7 @@
       </c>
       <c r="B362" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD | 19mm (0.75 in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C362" s="14" t="n"/>
@@ -29993,7 +30003,7 @@
       </c>
       <c r="B364" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD | 25.4mm (1 in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C364" s="14" t="n"/>
@@ -30040,7 +30050,7 @@
       </c>
       <c r="B366" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-RL | 330mm (13in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C366" s="14" t="n"/>
@@ -30087,7 +30097,7 @@
       </c>
       <c r="B368" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-Black | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C368" s="14" t="n"/>
@@ -30134,7 +30144,7 @@
       </c>
       <c r="B370" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 55mm (2.17") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C370" s="14" t="n"/>
@@ -30181,7 +30191,7 @@
       </c>
       <c r="B372" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 100mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C372" s="14" t="n"/>
@@ -30228,7 +30238,7 @@
       </c>
       <c r="B374" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 9.52mm (3/8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C374" s="14" t="n"/>
@@ -30275,7 +30285,7 @@
       </c>
       <c r="B376" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2SD | 38.1mm (1.5 in) wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C376" s="14" t="n"/>
@@ -30322,7 +30332,7 @@
       </c>
       <c r="B378" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-Black | 304.8mm (12") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C378" s="14" t="n"/>
@@ -30369,7 +30379,7 @@
       </c>
       <c r="B380" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-UT | 100mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C380" s="14" t="n"/>
@@ -30416,7 +30426,7 @@
       </c>
       <c r="B382" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-UT | 12.7mm (½") wide x 33m (36 yd) long</t>
         </is>
       </c>
       <c r="C382" s="14" t="n"/>
@@ -30463,7 +30473,7 @@
       </c>
       <c r="B384" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-UT | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C384" s="14" t="n"/>
@@ -30510,7 +30520,7 @@
       </c>
       <c r="B386" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-UT | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C386" s="14" t="n"/>
@@ -30557,7 +30567,7 @@
       </c>
       <c r="B388" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-UT | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C388" s="14" t="n"/>
@@ -30604,7 +30614,7 @@
       </c>
       <c r="B390" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-UT | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C390" s="14" t="n"/>
@@ -30651,7 +30661,7 @@
       </c>
       <c r="B392" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3N | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C392" s="14" t="n"/>
@@ -30698,7 +30708,7 @@
       </c>
       <c r="B394" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3N | 12.7mm (1/2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C394" s="14" t="n"/>
@@ -30745,7 +30755,7 @@
       </c>
       <c r="B396" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3N | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C396" s="14" t="n"/>
@@ -30792,7 +30802,7 @@
       </c>
       <c r="B398" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1AD-2RL | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C398" s="14" t="n"/>
@@ -30839,7 +30849,7 @@
       </c>
       <c r="B400" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1AD-2RL | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C400" s="14" t="n"/>
@@ -30886,7 +30896,7 @@
       </c>
       <c r="B402" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1AD-2RL | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C402" s="14" t="n"/>
@@ -30933,7 +30943,7 @@
       </c>
       <c r="B404" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1AD-2RL | 101.6mm (4") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C404" s="14" t="n"/>
@@ -30980,7 +30990,7 @@
       </c>
       <c r="B406" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 300mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C406" s="14" t="n"/>
@@ -31027,7 +31037,7 @@
       </c>
       <c r="B408" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-ALUM | 152.4mm (6") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C408" s="14" t="n"/>
@@ -31074,7 +31084,7 @@
       </c>
       <c r="B410" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-2RL | 305mm (12") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C410" s="14" t="n"/>
@@ -31121,7 +31131,7 @@
       </c>
       <c r="B412" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C412" s="14" t="n"/>
@@ -31168,7 +31178,7 @@
       </c>
       <c r="B414" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 305mm (12") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C414" s="14" t="n"/>
@@ -31215,7 +31225,7 @@
       </c>
       <c r="B416" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2SD | 60mm (2") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C416" s="14" t="n"/>
@@ -31262,7 +31272,7 @@
       </c>
       <c r="B418" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-FR | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C418" s="14" t="n"/>
@@ -31309,7 +31319,7 @@
       </c>
       <c r="B420" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-FR | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C420" s="14" t="n"/>
@@ -31356,7 +31366,7 @@
       </c>
       <c r="B422" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-FR | 19mm (¾") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C422" s="14" t="n"/>
@@ -31403,7 +31413,7 @@
       </c>
       <c r="B424" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-FR | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C424" s="14" t="n"/>
@@ -31450,7 +31460,7 @@
       </c>
       <c r="B426" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-FR | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C426" s="14" t="n"/>
@@ -31497,7 +31507,7 @@
       </c>
       <c r="B428" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 37mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C428" s="14" t="n"/>
@@ -31544,7 +31554,7 @@
       </c>
       <c r="B430" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-Black | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C430" s="14" t="n"/>
@@ -31591,7 +31601,7 @@
       </c>
       <c r="B432" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-Black | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C432" s="14" t="n"/>
@@ -31638,7 +31648,7 @@
       </c>
       <c r="B434" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-FR | 5.08mm (0.2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C434" s="14" t="n"/>
@@ -31685,7 +31695,7 @@
       </c>
       <c r="B436" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-ALUM | 10mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C436" s="14" t="n"/>
@@ -31732,7 +31742,7 @@
       </c>
       <c r="B438" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-ALUM | 100mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C438" s="14" t="n"/>
@@ -31779,7 +31789,7 @@
       </c>
       <c r="B440" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 9.5mm (⅜") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C440" s="14" t="n"/>
@@ -31826,7 +31836,7 @@
       </c>
       <c r="B442" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-RL | 305mm (12.01") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C442" s="14" t="n"/>
@@ -31873,7 +31883,7 @@
       </c>
       <c r="B444" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-FEP616 | 100mm (3.94") wide x 33m(36yd) long</t>
         </is>
       </c>
       <c r="C444" s="14" t="n"/>
@@ -31920,7 +31930,7 @@
       </c>
       <c r="B446" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-FEP019 | 100.0mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C446" s="14" t="n"/>
@@ -31967,7 +31977,7 @@
       </c>
       <c r="B448" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-FEP919 | 100.0mm (3.94") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C448" s="14" t="n"/>
@@ -32014,7 +32024,7 @@
       </c>
       <c r="B450" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 3.17mm (1/8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C450" s="14" t="n"/>
@@ -32061,7 +32071,7 @@
       </c>
       <c r="B452" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 3.97mm (5/32") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C452" s="14" t="n"/>
@@ -32108,7 +32118,7 @@
       </c>
       <c r="B454" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 4.76mm (3/16) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C454" s="14" t="n"/>
@@ -32155,7 +32165,7 @@
       </c>
       <c r="B456" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 380.0 mm (15") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C456" s="14" t="n"/>
@@ -32202,7 +32212,7 @@
       </c>
       <c r="B458" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N | 159mm (6.25") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C458" s="14" t="n"/>
@@ -32249,7 +32259,7 @@
       </c>
       <c r="B460" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1SD-2RL | 76.2mm (3") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C460" s="14" t="n"/>
@@ -32296,7 +32306,7 @@
       </c>
       <c r="B462" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1A-Yellow | 6.4mm (¼") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C462" s="14" t="n"/>
@@ -32343,7 +32353,7 @@
       </c>
       <c r="B464" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 70mm (2.75") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C464" s="14" t="n"/>
@@ -32390,7 +32400,7 @@
       </c>
       <c r="B466" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S | 70mm (2.75") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C466" s="14" t="n"/>
@@ -32437,7 +32447,7 @@
       </c>
       <c r="B468" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 70mm (2.75") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C468" s="14" t="n"/>
@@ -32484,7 +32494,7 @@
       </c>
       <c r="B470" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2AD | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C470" s="14" t="n"/>
@@ -32531,7 +32541,7 @@
       </c>
       <c r="B472" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD | 3 mm (0.12 in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C472" s="14" t="n"/>
@@ -32578,7 +32588,7 @@
       </c>
       <c r="B474" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD | 75 mm (2.95 in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C474" s="14" t="n"/>
@@ -32625,7 +32635,7 @@
       </c>
       <c r="B476" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3N | 38.1mm (1.5") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C476" s="14" t="n"/>
@@ -32672,7 +32682,7 @@
       </c>
       <c r="B478" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 7.5mm (0.3") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C478" s="14" t="n"/>
@@ -32719,7 +32729,7 @@
       </c>
       <c r="B480" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-DCD | 12.7mm (1/2 inch) diameter die cut discs - 2000 pcs</t>
         </is>
       </c>
       <c r="C480" s="14" t="n"/>
@@ -32766,7 +32776,7 @@
       </c>
       <c r="B482" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-DCD | 12.7mm (1/2inch) diameter die cut discs</t>
         </is>
       </c>
       <c r="C482" s="14" t="n"/>
@@ -32813,7 +32823,7 @@
       </c>
       <c r="B484" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD-DCD | 12.7mm (1/2inch) diameter die cut discs</t>
         </is>
       </c>
       <c r="C484" s="14" t="n"/>
@@ -32860,7 +32870,7 @@
       </c>
       <c r="B486" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S-DCD | 12.7mm (1/2inch) diameter die cut discs</t>
         </is>
       </c>
       <c r="C486" s="14" t="n"/>
@@ -32907,7 +32917,7 @@
       </c>
       <c r="B488" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 210mm (8.3") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C488" s="14" t="n"/>
@@ -32954,7 +32964,7 @@
       </c>
       <c r="B490" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-Clear | 8mm (0.3") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C490" s="14" t="n"/>
@@ -33001,7 +33011,7 @@
       </c>
       <c r="B492" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 3.2mm (1/8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C492" s="14" t="n"/>
@@ -33048,7 +33058,7 @@
       </c>
       <c r="B494" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 36.5mm (1.44") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C494" s="14" t="n"/>
@@ -33095,7 +33105,7 @@
       </c>
       <c r="B496" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 36.5mm (1.44") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C496" s="14" t="n"/>
@@ -33142,7 +33152,7 @@
       </c>
       <c r="B498" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 20.3mm (0.8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C498" s="14" t="n"/>
@@ -33189,7 +33199,7 @@
       </c>
       <c r="B500" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-Blue-DCD | 12.7mm (1/2 inch) diameter die cut discs - 2000 pcs</t>
         </is>
       </c>
       <c r="C500" s="14" t="n"/>
@@ -33236,7 +33246,7 @@
       </c>
       <c r="B502" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET2S-Blue-DCD | 12.7mm (1/2 inch) diameter die cut discs - 2000 pcs</t>
         </is>
       </c>
       <c r="C502" s="14" t="n"/>
@@ -33283,7 +33293,7 @@
       </c>
       <c r="B504" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 7.94mm (5/16") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C504" s="14" t="n"/>
@@ -33330,7 +33340,7 @@
       </c>
       <c r="B506" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-RL | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C506" s="14" t="n"/>
@@ -33377,7 +33387,7 @@
       </c>
       <c r="B508" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-RL | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C508" s="14" t="n"/>
@@ -33424,7 +33434,7 @@
       </c>
       <c r="B510" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 254mm (10") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C510" s="14" t="n"/>
@@ -33471,7 +33481,7 @@
       </c>
       <c r="B512" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 22mm (0.87") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C512" s="14" t="n"/>
@@ -33518,7 +33528,7 @@
       </c>
       <c r="B514" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S | 22mm (0.87") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C514" s="14" t="n"/>
@@ -33565,7 +33575,7 @@
       </c>
       <c r="B516" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 150mm (5.91") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C516" s="14" t="n"/>
@@ -33612,7 +33622,7 @@
       </c>
       <c r="B518" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 300mm (11.81") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C518" s="14" t="n"/>
@@ -33659,7 +33669,7 @@
       </c>
       <c r="B520" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S | 450mm (18") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C520" s="14" t="n"/>
@@ -33706,7 +33716,7 @@
       </c>
       <c r="B522" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-DCD | 6.4mm (1/4 inch) diameter die cut discs - 2000 pcs</t>
         </is>
       </c>
       <c r="C522" s="14" t="n"/>
@@ -33753,7 +33763,7 @@
       </c>
       <c r="B524" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 230.0 mm (9 1/16") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C524" s="14" t="n"/>
@@ -33800,7 +33810,7 @@
       </c>
       <c r="B526" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 50mm (1.97") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C526" s="14" t="n"/>
@@ -33847,7 +33857,7 @@
       </c>
       <c r="B528" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 81.3mm (3.2") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C528" s="14" t="n"/>
@@ -33894,7 +33904,7 @@
       </c>
       <c r="B530" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 112mm (4.4") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C530" s="14" t="n"/>
@@ -33941,7 +33951,7 @@
       </c>
       <c r="B532" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2N | 210mm (8.27") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C532" s="14" t="n"/>
@@ -33988,7 +33998,7 @@
       </c>
       <c r="B534" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3N | 210mm (8.27") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C534" s="14" t="n"/>
@@ -34035,7 +34045,7 @@
       </c>
       <c r="B536" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 9.12mm (0.36") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C536" s="14" t="n"/>
@@ -34082,7 +34092,7 @@
       </c>
       <c r="B538" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 6.73mm (0.26") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C538" s="14" t="n"/>
@@ -34129,7 +34139,7 @@
       </c>
       <c r="B540" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-Black | 12.7mm (0.5") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C540" s="14" t="n"/>
@@ -34176,7 +34186,7 @@
       </c>
       <c r="B542" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N-ALUM | 300mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C542" s="14" t="n"/>
@@ -34223,7 +34233,7 @@
       </c>
       <c r="B544" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-DCD | 100mm (3.93inch) diameter die cut discs</t>
         </is>
       </c>
       <c r="C544" s="14" t="n"/>
@@ -34270,7 +34280,7 @@
       </c>
       <c r="B546" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 50.8mm (2") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C546" s="14" t="n"/>
@@ -34317,7 +34327,7 @@
       </c>
       <c r="B548" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5N-DCD | 12.7mm (1/2inch) diameter die cut discs</t>
         </is>
       </c>
       <c r="C548" s="14" t="n"/>
@@ -34364,7 +34374,7 @@
       </c>
       <c r="B550" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 30mm (1.18") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C550" s="14" t="n"/>
@@ -34411,7 +34421,7 @@
       </c>
       <c r="B552" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 40mm (1.57") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C552" s="14" t="n"/>
@@ -34458,7 +34468,7 @@
       </c>
       <c r="B554" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 60mm (2.3") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C554" s="14" t="n"/>
@@ -34505,7 +34515,7 @@
       </c>
       <c r="B556" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5SD-UT-RL | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C556" s="14" t="n"/>
@@ -34552,7 +34562,7 @@
       </c>
       <c r="B558" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5SD-UT-RL | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C558" s="14" t="n"/>
@@ -34599,7 +34609,7 @@
       </c>
       <c r="B560" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5SD-UT-RL | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C560" s="14" t="n"/>
@@ -34646,7 +34656,7 @@
       </c>
       <c r="B562" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2AD | 50.8mm (2in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C562" s="14" t="n"/>
@@ -34693,7 +34703,7 @@
       </c>
       <c r="B564" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 15mm (0.6") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C564" s="14" t="n"/>
@@ -34740,7 +34750,7 @@
       </c>
       <c r="B566" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 114mm (4.48") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C566" s="14" t="n"/>
@@ -34787,7 +34797,7 @@
       </c>
       <c r="B568" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 116mm (4.56") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C568" s="14" t="n"/>
@@ -34834,7 +34844,7 @@
       </c>
       <c r="B570" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-T-RL | 254mm (10") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C570" s="14" t="n"/>
@@ -34881,7 +34891,7 @@
       </c>
       <c r="B572" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-T-RL | 50.8mm (2") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C572" s="14" t="n"/>
@@ -34928,7 +34938,7 @@
       </c>
       <c r="B574" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-T-RL | 114mm (4.48") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C574" s="14" t="n"/>
@@ -34975,7 +34985,7 @@
       </c>
       <c r="B576" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5N | 4.76mm (0.19") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C576" s="14" t="n"/>
@@ -35022,7 +35032,7 @@
       </c>
       <c r="B578" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 114mm (4.48") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C578" s="14" t="n"/>
@@ -35069,7 +35079,7 @@
       </c>
       <c r="B580" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-UT-RL | 50.8mm (2") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C580" s="14" t="n"/>
@@ -35116,7 +35126,7 @@
       </c>
       <c r="B582" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-UT-RL | 114mm (4.48") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C582" s="14" t="n"/>
@@ -35163,7 +35173,7 @@
       </c>
       <c r="B584" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2AD | 350mm wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C584" s="14" t="n"/>
@@ -35210,7 +35220,7 @@
       </c>
       <c r="B586" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 10mm (0.39") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C586" s="14" t="n"/>
@@ -35257,7 +35267,7 @@
       </c>
       <c r="B588" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 20mm (0.78") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C588" s="14" t="n"/>
@@ -35304,7 +35314,7 @@
       </c>
       <c r="B590" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 30mm (1.18") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C590" s="14" t="n"/>
@@ -35351,7 +35361,7 @@
       </c>
       <c r="B592" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD | 6.35mm (0.25 in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C592" s="14" t="n"/>
@@ -35398,7 +35408,7 @@
       </c>
       <c r="B594" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 9.52mm (3/8") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C594" s="14" t="n"/>
@@ -35445,7 +35455,7 @@
       </c>
       <c r="B596" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 11.11mm (0.44") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C596" s="14" t="n"/>
@@ -35492,7 +35502,7 @@
       </c>
       <c r="B598" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ALUM | 254mm (10") wide x 27.4m (30yd) long</t>
         </is>
       </c>
       <c r="C598" s="14" t="n"/>
@@ -35539,7 +35549,7 @@
       </c>
       <c r="B600" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5SD-UT-RL | 112mm (4.4") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C600" s="14" t="n"/>
@@ -35586,7 +35596,7 @@
       </c>
       <c r="B602" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5SD-UT-RL | 284mm (11.18") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C602" s="14" t="n"/>
@@ -35633,7 +35643,7 @@
       </c>
       <c r="B604" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3N | 152.4mm (6") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C604" s="14" t="n"/>
@@ -35680,7 +35690,7 @@
       </c>
       <c r="B606" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 5mm (0.19") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C606" s="14" t="n"/>
@@ -35727,7 +35737,7 @@
       </c>
       <c r="B608" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-T-RL | 44mm (1.73") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C608" s="14" t="n"/>
@@ -35774,7 +35784,7 @@
       </c>
       <c r="B610" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-LO | 355mm (14") wide x 27m (30yd) long</t>
         </is>
       </c>
       <c r="C610" s="14" t="n"/>
@@ -35821,7 +35831,7 @@
       </c>
       <c r="B612" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3S | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C612" s="14" t="n"/>
@@ -35868,7 +35878,7 @@
       </c>
       <c r="B614" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3S-RL | 114mm (4.5") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C614" s="14" t="n"/>
@@ -35915,7 +35925,7 @@
       </c>
       <c r="B616" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3S | 114mm (4.5") wide x 33m (36yd) long (Tolerance is ± 0.5" - 1.3cm)</t>
         </is>
       </c>
       <c r="C616" s="14" t="n"/>
@@ -35962,7 +35972,7 @@
       </c>
       <c r="B618" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 114mm (4.5") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C618" s="14" t="n"/>
@@ -36009,7 +36019,7 @@
       </c>
       <c r="B620" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3S-RL | 50mm (1.96") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C620" s="14" t="n"/>
@@ -36056,7 +36066,7 @@
       </c>
       <c r="B622" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-T-RL | 50.8mm (2") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C622" s="14" t="n"/>
@@ -36103,7 +36113,7 @@
       </c>
       <c r="B624" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-T-RL | 114mm (4.48") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C624" s="14" t="n"/>
@@ -36150,7 +36160,7 @@
       </c>
       <c r="B626" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3S-T-RL | 50.8mm (2") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C626" s="14" t="n"/>
@@ -36197,7 +36207,7 @@
       </c>
       <c r="B628" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3S-T-RL | 114mm (4.48") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C628" s="14" t="n"/>
@@ -36244,7 +36254,7 @@
       </c>
       <c r="B630" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-LO | 12.7mm (1/2") wide x 27m (30yd) long</t>
         </is>
       </c>
       <c r="C630" s="14" t="n"/>
@@ -36291,7 +36301,7 @@
       </c>
       <c r="B632" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-LO | 25.4mm (1") wide x 27m (30yd) long</t>
         </is>
       </c>
       <c r="C632" s="14" t="n"/>
@@ -36338,7 +36348,7 @@
       </c>
       <c r="B634" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-LO | 50.8mm (2") wide x 27.4m (30yd) long</t>
         </is>
       </c>
       <c r="C634" s="14" t="n"/>
@@ -36385,7 +36395,7 @@
       </c>
       <c r="B636" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-LO | 25.4mm (1") wide x 27.4m (30yd) long</t>
         </is>
       </c>
       <c r="C636" s="14" t="n"/>
@@ -36432,7 +36442,7 @@
       </c>
       <c r="B638" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S2-RL | 50.8mm (2") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C638" s="14" t="n"/>
@@ -36479,7 +36489,7 @@
       </c>
       <c r="B640" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S2-RL | 114mm (4.48") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C640" s="14" t="n"/>
@@ -36526,7 +36536,7 @@
       </c>
       <c r="B642" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-B | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C642" s="14" t="n"/>
@@ -36573,7 +36583,7 @@
       </c>
       <c r="B644" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S | 21.5mm (0.85") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C644" s="14" t="n"/>
@@ -36620,7 +36630,7 @@
       </c>
       <c r="B646" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2AD-LO | 355mm (14") wide x 27.5m (30yd) long</t>
         </is>
       </c>
       <c r="C646" s="14" t="n"/>
@@ -36667,7 +36677,7 @@
       </c>
       <c r="B648" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2AD-LO | 12.7mm (1/2") wide x 27.5m (30yd) long</t>
         </is>
       </c>
       <c r="C648" s="14" t="n"/>
@@ -36714,7 +36724,7 @@
       </c>
       <c r="B650" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2AD-LO | 25.4mm (1") wide x 27.5m (30yd) long</t>
         </is>
       </c>
       <c r="C650" s="14" t="n"/>
@@ -36761,7 +36771,7 @@
       </c>
       <c r="B652" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-Black | 152.4mm (6") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C652" s="14" t="n"/>
@@ -36808,7 +36818,7 @@
       </c>
       <c r="B654" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-BRL | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C654" s="14" t="n"/>
@@ -36855,7 +36865,7 @@
       </c>
       <c r="B656" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-BRL | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C656" s="14" t="n"/>
@@ -36902,7 +36912,7 @@
       </c>
       <c r="B658" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-BRL | 304.8mm (12") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C658" s="14" t="n"/>
@@ -36949,7 +36959,7 @@
       </c>
       <c r="B660" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-BRL | 12.7mm (0.5") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C660" s="14" t="n"/>
@@ -36996,7 +37006,7 @@
       </c>
       <c r="B662" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD-BRL | 152.4mm (6") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C662" s="14" t="n"/>
@@ -37043,7 +37053,7 @@
       </c>
       <c r="B664" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 63.5mm (2.5") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C664" s="14" t="n"/>
@@ -37090,7 +37100,7 @@
       </c>
       <c r="B666" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-T-RL | 162mm (6.37") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C666" s="14" t="n"/>
@@ -37137,7 +37147,7 @@
       </c>
       <c r="B668" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-T-RL | 162mm (6.37") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C668" s="14" t="n"/>
@@ -37184,7 +37194,7 @@
       </c>
       <c r="B670" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2S-RL | 162mm (6.37") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C670" s="14" t="n"/>
@@ -37231,7 +37241,7 @@
       </c>
       <c r="B672" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET2S-Green | 101.6mm (4 in) wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C672" s="14" t="n"/>
@@ -37278,7 +37288,7 @@
       </c>
       <c r="B674" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 3mm (0.12") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C674" s="14" t="n"/>
@@ -37325,7 +37335,7 @@
       </c>
       <c r="B676" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1A-Yellow | 32mm (1¼") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C676" s="14" t="n"/>
@@ -37372,7 +37382,7 @@
       </c>
       <c r="B678" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1A-Yellow | 28mm (1.1") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C678" s="14" t="n"/>
@@ -37419,7 +37429,7 @@
       </c>
       <c r="B680" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1A-Yellow | 26mm (1") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C680" s="14" t="n"/>
@@ -37466,7 +37476,7 @@
       </c>
       <c r="B682" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1A-Yellow | 17mm (⅔") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C682" s="14" t="n"/>
@@ -37513,7 +37523,7 @@
       </c>
       <c r="B684" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 254mm (10") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C684" s="14" t="n"/>
@@ -37560,7 +37570,7 @@
       </c>
       <c r="B686" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A | 60mm (2.36") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C686" s="14" t="n"/>
@@ -37607,7 +37617,7 @@
       </c>
       <c r="B688" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1A-Yellow | 50.8mm (2") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C688" s="14" t="n"/>
@@ -37654,7 +37664,7 @@
       </c>
       <c r="B690" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1A-Yellow | 38.1 mm (1½") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C690" s="14" t="n"/>
@@ -37701,7 +37711,7 @@
       </c>
       <c r="B692" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-T-RL | 164mm (6.46" ±0.5 mm) wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C692" s="14" t="n"/>
@@ -37748,7 +37758,7 @@
       </c>
       <c r="B694" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT3N | 14mm (0,55") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C694" s="14" t="n"/>
@@ -37795,7 +37805,7 @@
       </c>
       <c r="B696" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET2S-Green | 38mm (1 1/2 in) wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C696" s="14" t="n"/>
@@ -37842,7 +37852,7 @@
       </c>
       <c r="B698" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET2S-Green | 76mm (3 in) wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C698" s="14" t="n"/>
@@ -37889,7 +37899,7 @@
       </c>
       <c r="B700" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S-RL | 12.7mm (½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C700" s="14" t="n"/>
@@ -37936,7 +37946,7 @@
       </c>
       <c r="B702" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S-RL | 25.4mm (1") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C702" s="14" t="n"/>
@@ -37983,7 +37993,7 @@
       </c>
       <c r="B704" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT5S-RL | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C704" s="14" t="n"/>
@@ -38030,7 +38040,7 @@
       </c>
       <c r="B706" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-ESD | 200mm (7.87") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C706" s="14" t="n"/>
@@ -38077,7 +38087,7 @@
       </c>
       <c r="B708" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-WL-SG | 12mm (0.47") wide x 30m (33yd) long</t>
         </is>
       </c>
       <c r="C708" s="14" t="n"/>
@@ -38124,7 +38134,7 @@
       </c>
       <c r="B710" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A | 36.83mm (1.45") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C710" s="14" t="n"/>
@@ -38171,7 +38181,7 @@
       </c>
       <c r="B712" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-FRC | 12mm wide x 33m (36yd)</t>
         </is>
       </c>
       <c r="C712" s="14" t="n"/>
@@ -38218,7 +38228,7 @@
       </c>
       <c r="B714" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL | 70mm (2.75") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C714" s="14" t="n"/>
@@ -38265,7 +38275,7 @@
       </c>
       <c r="B716" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-UT | 38.1mm (1½") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C716" s="14" t="n"/>
@@ -38312,7 +38322,7 @@
       </c>
       <c r="B718" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-UT-RL | 100mm (3.93") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C718" s="14" t="n"/>
@@ -38359,7 +38369,7 @@
       </c>
       <c r="B720" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-Clear | 38.1mm (1.5") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C720" s="14" t="n"/>
@@ -38406,7 +38416,7 @@
       </c>
       <c r="B722" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-B | 50.8mm (2") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C722" s="14" t="n"/>
@@ -38453,7 +38463,7 @@
       </c>
       <c r="B724" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PET1S-UT-Clear | 38.1mm (1.5") wide x 66m (72yd) long</t>
         </is>
       </c>
       <c r="C724" s="14" t="n"/>
@@ -38500,7 +38510,7 @@
       </c>
       <c r="B726" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT | 200mm (7.87") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C726" s="14" t="n"/>
@@ -38547,7 +38557,7 @@
       </c>
       <c r="B728" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-T-RL | 62mm (2.4") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C728" s="14" t="n"/>
@@ -38594,7 +38604,7 @@
       </c>
       <c r="B730" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-UT-RL | 62mm (2.4") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C730" s="14" t="n"/>
@@ -38641,7 +38651,7 @@
       </c>
       <c r="B732" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-WL-SG | 100mm (3.94") wide x 100m (109yd) long</t>
         </is>
       </c>
       <c r="C732" s="14" t="n"/>
@@ -38688,7 +38698,7 @@
       </c>
       <c r="B734" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-LO | 400mm (15.7") wide x 27m (30yd) long</t>
         </is>
       </c>
       <c r="C734" s="14" t="n"/>
@@ -38735,7 +38745,7 @@
       </c>
       <c r="B736" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1A-LO | 400mm (15.7") wide x 27.4m (30yd) long</t>
         </is>
       </c>
       <c r="C736" s="14" t="n"/>
@@ -38782,7 +38792,7 @@
       </c>
       <c r="B738" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 4.3mm (0.169") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C738" s="14" t="n"/>
@@ -38829,7 +38839,7 @@
       </c>
       <c r="B740" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 160mm (6.30") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C740" s="14" t="n"/>
@@ -38876,7 +38886,7 @@
       </c>
       <c r="B742" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 200mm (7.78") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C742" s="14" t="n"/>
@@ -38923,7 +38933,7 @@
       </c>
       <c r="B744" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-B | 190mm (7.48") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C744" s="14" t="n"/>
@@ -38970,7 +38980,7 @@
       </c>
       <c r="B746" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL-Series | 140.13mm x 64.45mm (1 set 2 parts)</t>
         </is>
       </c>
       <c r="C746" s="14" t="n"/>
@@ -39017,7 +39027,7 @@
       </c>
       <c r="B748" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-RL-Series | 132.47 mm x 54.35 mm (1 set 2 parts)</t>
         </is>
       </c>
       <c r="C748" s="14" t="n"/>
@@ -39064,7 +39074,7 @@
       </c>
       <c r="B750" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-ESD-Series | 330 mm (12.992 in) wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C750" s="14" t="n"/>
@@ -39111,7 +39121,7 @@
       </c>
       <c r="B752" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT2A-FR Series | 65mm (22.24") wide x 33m (36 yd) long</t>
         </is>
       </c>
       <c r="C752" s="14" t="n"/>
@@ -39158,7 +39168,7 @@
       </c>
       <c r="B754" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT0.5S-UT-RL | 164mm (6.50") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C754" s="14" t="n"/>
@@ -39205,7 +39215,7 @@
       </c>
       <c r="B756" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1S-UT-RL | 164mm (6.5") wide x 33m (36yd) long with release liner</t>
         </is>
       </c>
       <c r="C756" s="14" t="n"/>
@@ -39252,7 +39262,7 @@
       </c>
       <c r="B758" s="14" t="inlineStr">
         <is>
-          <t>Outsourcing Charge</t>
+          <t>PIT1N | 164mm (6.5") wide x 33m (36yd) long</t>
         </is>
       </c>
       <c r="C758" s="14" t="n"/>

</xml_diff>